<commit_message>
refactor(briefs): promote SCUC inline headers to H2 subheadings
Convert all 21 corpus briefs from inline-bold (`**Situation.** Text…`)
to block subheadings (`## Situation` on its own line, body paragraph
beneath). H2 headers carry visual weight in any markdown context —
canvas, GitHub render, LinkedIn screen capture — so the SCUC bones
read as four distinct sections, not a subtle paragraph lead-in.

Skill updated to teach H2 subheadings as canonical SCUC form. Rubric
criteria unchanged (they assert content, not shape). corpus-content.xlsx
refreshed.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/corpus-content.xlsx
+++ b/experiments/corpus-content.xlsx
@@ -503,10 +503,14 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t># Apartment search for a renter with a past eviction — design exploration
-**Situation.** A person with an eviction record is looking for a new place to live. The eviction may have followed a job loss, a medical event, or a dispute with a prior landlord — sometimes a dismissed filing, sometimes a filing-in-error, sometimes a completed eviction-for-cause. The renter has since rebuilt: a job, references, money for a deposit. What reaches the landlord is a tenant-screening report — bundling rental, credit, employment, and criminal history into a score — on which the filing looks the same whether the case was won, lost, or dismissed.
-**Complication.** The renter pays application fees at every listing and discovers, sometimes days later, that they have been declined. They get back a vague "did not meet screening criteria" or no explanation at all. There is no path to find out which factor produced the decline, no path to contest a record they believe is inaccurate. They confront listing aggregators, screening companies whose reports they cannot see, bureau disputes that move slowly, and legal-aid offices whose capacity does not meet the volume.
-**Users.** The renter with the eviction record on their file. Landlords and screening companies are stakeholders, not the target — the design is for the renter with weeks, not months, and a stack of declined applications. Scope is "I'm looking" through "I've signed a lease."
-**Cost.** They need to be housed in the weeks they have, not the months a dispute would take. Fees stack up against a deposit they are trying to keep intact. Each decline arrives without enough information to act on, and the next listing goes up against the same report. The current housing is running out or already gone.</t>
+## Situation
+A person with an eviction record is looking for a new place to live. The eviction may have followed a job loss, a medical event, or a dispute with a prior landlord — sometimes a dismissed filing, sometimes a filing-in-error, sometimes a completed eviction-for-cause. The renter has since rebuilt: a job, references, money for a deposit. What reaches the landlord is a tenant-screening report — bundling rental, credit, employment, and criminal history into a score — on which the filing looks the same whether the case was won, lost, or dismissed.
+## Complication
+The renter pays application fees at every listing and discovers, sometimes days later, that they have been declined. They get back a vague "did not meet screening criteria" or no explanation at all. There is no path to find out which factor produced the decline, no path to contest a record they believe is inaccurate. They confront listing aggregators, screening companies whose reports they cannot see, bureau disputes that move slowly, and legal-aid offices whose capacity does not meet the volume.
+## Users
+The renter with the eviction record on their file. Landlords and screening companies are stakeholders, not the target — the design is for the renter with weeks, not months, and a stack of declined applications. Scope is "I'm looking" through "I've signed a lease."
+## Cost
+They need to be housed in the weeks they have, not the months a dispute would take. Fees stack up against a deposit they are trying to keep intact. Each decline arrives without enough information to act on, and the next listing goes up against the same report. The current housing is running out or already gone.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -562,10 +566,14 @@
       <c r="B3" s="3" t="inlineStr">
         <is>
           <t># Coordinating care for an aging parent — design exploration
-**Situation.** An adult child is responsible for the day-to-day care of an aging parent in another city. They are working full-time, may be raising their own kids, and are now also managing their parent's medications, appointments, insurance disputes, in-home aide schedule, finances, and longer-term decisions about home modifications, assisted living, or hospice — with sibling involvement that ranges from supportive to fractious.
-**Complication.** The information lives everywhere — their own phone, their email, the parent's hand-written notes on a yellow pad by the kitchen phone, the parent's doctor's portals (three or four, each with its own login), Medicare statements, the aide's notebook, the pharmacy's text messages. No system holds the picture; the caregiver holds it, in their head, between work meetings and bedtime. The new prescription started last Thursday is supposed to be checked against the cardiologist's older one that may or may not have been discontinued. The PCP's portal does not show the cardiologist's prescriptions. The aide's notebook is three hundred miles away.
-**Users.** The adult-child caregiver and the aging parent, as a dyad — the parent in their own apartment, the caregiver coordinating from three hundred miles away. Siblings, aides, doctors, and pharmacists are stakeholders the design accommodates, not optimizes for. Scope is the rhythm of a month, not a single appointment.
-**Cost.** When something goes wrong — a missed medication, a duplicate dose, an ED visit that looks preventable in hindsight — the gap was between systems the caregiver was supposed to bridge across. The parent absorbs the errors when the picture slips. The work eats evenings, weekends, and the bandwidth left for everything else in the caregiver's life.</t>
+## Situation
+An adult child is responsible for the day-to-day care of an aging parent in another city. They are working full-time, may be raising their own kids, and are now also managing their parent's medications, appointments, insurance disputes, in-home aide schedule, finances, and longer-term decisions about home modifications, assisted living, or hospice — with sibling involvement that ranges from supportive to fractious.
+## Complication
+The information lives everywhere — their own phone, their email, the parent's hand-written notes on a yellow pad by the kitchen phone, the parent's doctor's portals (three or four, each with its own login), Medicare statements, the aide's notebook, the pharmacy's text messages. No system holds the picture; the caregiver holds it, in their head, between work meetings and bedtime. The new prescription started last Thursday is supposed to be checked against the cardiologist's older one that may or may not have been discontinued. The PCP's portal does not show the cardiologist's prescriptions. The aide's notebook is three hundred miles away.
+## Users
+The adult-child caregiver and the aging parent, as a dyad — the parent in their own apartment, the caregiver coordinating from three hundred miles away. Siblings, aides, doctors, and pharmacists are stakeholders the design accommodates, not optimizes for. Scope is the rhythm of a month, not a single appointment.
+## Cost
+When something goes wrong — a missed medication, a duplicate dose, an ED visit that looks preventable in hindsight — the gap was between systems the caregiver was supposed to bridge across. The parent absorbs the errors when the picture slips. The work eats evenings, weekends, and the bandwidth left for everything else in the caregiver's life.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -621,10 +629,14 @@
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t># An adult learner re-entering community college — design exploration
-**Situation.** An adult — twenty-five, thirty-five, fifty — has enrolled at community college, often after years away from formal schooling. They've decided to re-enroll for a new credential, an industry switch, or developmental coursework before a four-year transfer. They've signed up; they haven't started. They have a job that won't easily flex, kids who need pick-up, and the cognitive disjuncture of being asked to think like a student again after years of not being one.
-**Complication.** They are trying to read a college website built for eighteen-year-olds applying for fall. They are unsure where to park, what to bring to orientation, whether the FAFSA they filled out applies to summer term, whether they can register part-time without losing the financial-aid bracket, and how to reach an advisor who answers in less than two weeks.
-**Users.** The adult learner re-entering community college after years away — not the eighteen-year-old applying for fall, and not the returner with a working campus rhythm. Advisors, financial-aid officers, and registrars are stakeholders the design encounters, not optimizes for. Scope is the eight-week window from "I've enrolled" through "I've completed the first month of classes."
-**Cost.** The first month is where the workable rhythm either gets built or doesn't. When the answers don't arrive in the window — when orientation feels alien, when the FAFSA question goes two weeks without a reply, when the parking and pick-up logistics don't line up — the learner quietly stops coming. The enrollment becomes another unfinished credential, the tuition becomes a sunk cost, and the next attempt is years out.</t>
+## Situation
+An adult — twenty-five, thirty-five, fifty — has enrolled at community college, often after years away from formal schooling. They've decided to re-enroll for a new credential, an industry switch, or developmental coursework before a four-year transfer. They've signed up; they haven't started. They have a job that won't easily flex, kids who need pick-up, and the cognitive disjuncture of being asked to think like a student again after years of not being one.
+## Complication
+They are trying to read a college website built for eighteen-year-olds applying for fall. They are unsure where to park, what to bring to orientation, whether the FAFSA they filled out applies to summer term, whether they can register part-time without losing the financial-aid bracket, and how to reach an advisor who answers in less than two weeks.
+## Users
+The adult learner re-entering community college after years away — not the eighteen-year-old applying for fall, and not the returner with a working campus rhythm. Advisors, financial-aid officers, and registrars are stakeholders the design encounters, not optimizes for. Scope is the eight-week window from "I've enrolled" through "I've completed the first month of classes."
+## Cost
+The first month is where the workable rhythm either gets built or doesn't. When the answers don't arrive in the window — when orientation feels alien, when the FAFSA question goes two weeks without a reply, when the parking and pick-up logistics don't line up — the learner quietly stops coming. The enrollment becomes another unfinished credential, the tuition becomes a sunk cost, and the next attempt is years out.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -679,10 +691,14 @@
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t># Disputing a credit-report error — design exploration
-**Situation.** A person has been denied an apartment, a job, a loan, or an insurance rate because of something on their credit report — and the something is wrong. A debt they paid years ago. An account opened in their name fraudulently. Identity confusion with a relative who shares their name. They have proof — receipts, closure letters, identity-theft affidavits — and no clear path to get it to the right place.
-**Complication.** They face three different dispute interfaces, one per bureau, each demanding documentation in slightly different formats and each capable of returning a one-line "investigated, no change" weeks later. They are unsure whether to write a paper letter, use the online portals, file directly with the furnisher, file a CFPB complaint, or do all four. The original error often reappears later from a different furnisher, and the consumer is back at the same three logins, the same documentation queue, the same wait. They confront the bureaus' portals, free-credit-report sites that funnel toward paid monitoring, the CFPB channel, IdentityTheft.gov, and legal-aid whose capacity does not meet the volume.
-**Users.** The consumer disputing the error — the one with receipts and closure letters in hand. Bureaus, furnishers, and CFPB intake staff are stakeholders, not the target. Scope is from noticing the error through resolution.
-**Cost.** The process unfolds over thirty to ninety days while the apartment application sits in limbo and the new job offer is on hold. The denial that prompted the dispute does not pause for resolution. When the error reappears from a different furnisher, the consumer is back at the same three logins, doing the work again on a life that has moved on.</t>
+## Situation
+A person has been denied an apartment, a job, a loan, or an insurance rate because of something on their credit report — and the something is wrong. A debt they paid years ago. An account opened in their name fraudulently. Identity confusion with a relative who shares their name. They have proof — receipts, closure letters, identity-theft affidavits — and no clear path to get it to the right place.
+## Complication
+They face three different dispute interfaces, one per bureau, each demanding documentation in slightly different formats and each capable of returning a one-line "investigated, no change" weeks later. They are unsure whether to write a paper letter, use the online portals, file directly with the furnisher, file a CFPB complaint, or do all four. The original error often reappears later from a different furnisher, and the consumer is back at the same three logins, the same documentation queue, the same wait. They confront the bureaus' portals, free-credit-report sites that funnel toward paid monitoring, the CFPB channel, IdentityTheft.gov, and legal-aid whose capacity does not meet the volume.
+## Users
+The consumer disputing the error — the one with receipts and closure letters in hand. Bureaus, furnishers, and CFPB intake staff are stakeholders, not the target. Scope is from noticing the error through resolution.
+## Cost
+The process unfolds over thirty to ninety days while the apartment application sits in limbo and the new job offer is on hold. The denial that prompted the dispute does not pause for resolution. When the error reappears from a different furnisher, the consumer is back at the same three logins, doing the work again on a life that has moved on.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -737,10 +753,14 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t># First contact with 988, the crisis line — design exploration
-**Situation.** Someone is reaching out to the US crisis line — 988 — for the first time. They may be experiencing a suicidal crisis, an acute panic episode, a substance-use crisis, or distress around grief, abuse, or identity. They may be the person in crisis, or a friend or family member trying to help someone else. They are reaching out at a moment of acute vulnerability and have a choice to make about whether to stay on the line.
-**Complication.** The first sixty seconds are determinative. What does this look like; will I be judged; what's about to happen; will police be sent to my address if I say the wrong thing. People who have heard that police might be dispatched are hesitant in ways the system has to meet; people who have never reached out before are calibrating from the screen, the voice, the hold music. The decision to keep reaching, or to hang up and not try again, is made before anyone has said anything.
-**Users.** The first-time reacher — the person in crisis, or the friend or family member calling on their behalf — in the opening seconds before a counselor has spoken. Counselors and dispatchers are stakeholders the design hands off to, not optimizes for. Scope is the call, text, or chat opening plus the immediate next step; the counselor protocol itself is out of scope.
-**Cost.** When the first sixty seconds don't hold, the person hangs up and does not try again. The next acute moment arrives without a line they trust. The friend who was calling for someone else goes back with nothing to offer.</t>
+## Situation
+Someone is reaching out to the US crisis line — 988 — for the first time. They may be experiencing a suicidal crisis, an acute panic episode, a substance-use crisis, or distress around grief, abuse, or identity. They may be the person in crisis, or a friend or family member trying to help someone else. They are reaching out at a moment of acute vulnerability and have a choice to make about whether to stay on the line.
+## Complication
+The first sixty seconds are determinative. What does this look like; will I be judged; what's about to happen; will police be sent to my address if I say the wrong thing. People who have heard that police might be dispatched are hesitant in ways the system has to meet; people who have never reached out before are calibrating from the screen, the voice, the hold music. The decision to keep reaching, or to hang up and not try again, is made before anyone has said anything.
+## Users
+The first-time reacher — the person in crisis, or the friend or family member calling on their behalf — in the opening seconds before a counselor has spoken. Counselors and dispatchers are stakeholders the design hands off to, not optimizes for. Scope is the call, text, or chat opening plus the immediate next step; the counselor protocol itself is out of scope.
+## Cost
+When the first sixty seconds don't hold, the person hangs up and does not try again. The next acute moment arrives without a line they trust. The friend who was calling for someone else goes back with nothing to offer.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -794,10 +814,14 @@
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t># Closing a deceased family member's accounts — design exploration
-**Situation.** When a person dies, someone in the family inherits an administrative ordeal nobody trained them for. They are the executor — spouse, adult child, sibling — and now need to identify, contact, and close out dozens of accounts: banks, credit cards, utilities, mortgages, retirement accounts, insurance, Social Security, and a digital life of email and photos and subscriptions. They are doing this in the evenings, between the funeral and the rest of life — often from a different city than the deceased, with a death certificate in hand and a stack of unopened mail.
-**Complication.** Each institution has its own forms, its own definitions, its own staff. Debt collectors begin calling within days; most are wrong about what the survivor owes, but the conversations are intimidating and the rules vary by state. The available resources are accurate and encyclopedic; they list eighty things the executor might need to do, with no way to know which twelve apply today.
-**Users.** The executor — spouse, adult child, or sibling — grieving and doing this because someone had to be. Institutions and debt collectors are stakeholders, not the design's target. Scope is from the first week through final dissolution.
-**Cost.** The work runs in the evenings on top of grief, on top of a job, on top of a household that did not pause. The encyclopedic list does not tell the executor which twelve of eighty steps belong to today, so the wrong ones get done first or none at all. The collectors' calls keep coming. The estate stays open, the mail keeps arriving, and the grief is interrupted every time the ordeal reasserts itself.</t>
+## Situation
+When a person dies, someone in the family inherits an administrative ordeal nobody trained them for. They are the executor — spouse, adult child, sibling — and now need to identify, contact, and close out dozens of accounts: banks, credit cards, utilities, mortgages, retirement accounts, insurance, Social Security, and a digital life of email and photos and subscriptions. They are doing this in the evenings, between the funeral and the rest of life — often from a different city than the deceased, with a death certificate in hand and a stack of unopened mail.
+## Complication
+Each institution has its own forms, its own definitions, its own staff. Debt collectors begin calling within days; most are wrong about what the survivor owes, but the conversations are intimidating and the rules vary by state. The available resources are accurate and encyclopedic; they list eighty things the executor might need to do, with no way to know which twelve apply today.
+## Users
+The executor — spouse, adult child, or sibling — grieving and doing this because someone had to be. Institutions and debt collectors are stakeholders, not the design's target. Scope is from the first week through final dissolution.
+## Cost
+The work runs in the evenings on top of grief, on top of a job, on top of a household that did not pause. The encyclopedic list does not tell the executor which twelve of eighty steps belong to today, so the wrong ones get done first or none at all. The collectors' calls keep coming. The estate stays open, the mail keeps arriving, and the grief is interrupted every time the ordeal reasserts itself.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -851,10 +875,14 @@
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t># Driver's license transfer after a cross-state move — design exploration
-**Situation.** A person has moved from one US state to another. They have a job to start, an apartment to unpack, a kid in a new school. Somewhere on the list is "transfer the driver's license," and the new state's DMV site is a tangle of pages that don't quite match the user's situation: out-of-state transfer vs new resident vs non-citizen vs recently-licensed teen. They have a stack of documents — birth certificate, Social Security card, lease, utility bill, old license, marriage certificate.
-**Complication.** They aren't sure which documents the office will accept on the day. They want to know when to go, what to bring, what the visit will feel like, and what happens if something goes wrong. The DMV won't tell them ahead of time. The mover does the visit, leaves with a temporary paper printout, and waits weeks for the hard copy in the mail. In the meantime they aren't sure whether the paper is enough to fly, open a bank account, or pass any other ID check.
-**Users.** A recent mover in the four-to-six-week window after a cross-state move, navigating the new state's DMV alone with a folder of documents and other life on fire.
-**Cost.** Getting any of this wrong costs another visit, another day of work missed, and the same lack of information about what's next. The scope is the four-to-six-week window after a move during which the license needs to transfer.</t>
+## Situation
+A person has moved from one US state to another. They have a job to start, an apartment to unpack, a kid in a new school. Somewhere on the list is "transfer the driver's license," and the new state's DMV site is a tangle of pages that don't quite match the user's situation: out-of-state transfer vs new resident vs non-citizen vs recently-licensed teen. They have a stack of documents — birth certificate, Social Security card, lease, utility bill, old license, marriage certificate.
+## Complication
+They aren't sure which documents the office will accept on the day. They want to know when to go, what to bring, what the visit will feel like, and what happens if something goes wrong. The DMV won't tell them ahead of time. The mover does the visit, leaves with a temporary paper printout, and waits weeks for the hard copy in the mail. In the meantime they aren't sure whether the paper is enough to fly, open a bank account, or pass any other ID check.
+## Users
+A recent mover in the four-to-six-week window after a cross-state move, navigating the new state's DMV alone with a folder of documents and other life on fire.
+## Cost
+Getting any of this wrong costs another visit, another day of work missed, and the same lack of information about what's next. The scope is the four-to-six-week window after a move during which the license needs to transfer.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -907,10 +935,14 @@
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t># A first-time manager's first performance review — design exploration
-**Situation.** Someone who has been a people manager for less than a year sits down at midnight to write their first performance review of an employee. They have nine weeks of notes — most of them mental — and a template HR handed down with fifteen sections and a five-point rating scale. They are also navigating a calibration cycle in which their ratings will be compared against peer managers' ratings, with rules they only half-understand.
-**Complication.** The performance-management software they're using delivers prompts and templates but does not actually help them think through what to say to this specific person about this specific thing. They are scared of doing harm. Of giving feedback that lands wrong. Of being too soft and ducking the real issue. Of being too critical and damaging a working relationship. They are alone with a form and a blinking cursor.
-**Users.** A first-time people manager writing their first review of a direct report — who might be a former peer, someone they hired, or someone with more years in the industry than they have. HR and the calibration committee are stakeholders the manager has to satisfy, but the design is for the manager in the moment of writing.
-**Cost.** The cost of getting this wrong is paid both at the next 1:1 and across the year that follows — a damaged working relationship, a real issue ducked, or feedback that lands so wrong it forecloses growth. The scope is the act of writing the review — the hours between *I have to write this* and *I have a draft I'd send.*</t>
+## Situation
+Someone who has been a people manager for less than a year sits down at midnight to write their first performance review of an employee. They have nine weeks of notes — most of them mental — and a template HR handed down with fifteen sections and a five-point rating scale. They are also navigating a calibration cycle in which their ratings will be compared against peer managers' ratings, with rules they only half-understand.
+## Complication
+The performance-management software they're using delivers prompts and templates but does not actually help them think through what to say to this specific person about this specific thing. They are scared of doing harm. Of giving feedback that lands wrong. Of being too soft and ducking the real issue. Of being too critical and damaging a working relationship. They are alone with a form and a blinking cursor.
+## Users
+A first-time people manager writing their first review of a direct report — who might be a former peer, someone they hired, or someone with more years in the industry than they have. HR and the calibration committee are stakeholders the manager has to satisfy, but the design is for the manager in the moment of writing.
+## Cost
+The cost of getting this wrong is paid both at the next 1:1 and across the year that follows — a damaged working relationship, a real issue ducked, or feedback that lands so wrong it forecloses growth. The scope is the act of writing the review — the hours between *I have to write this* and *I have a draft I'd send.*</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -964,10 +996,14 @@
       <c r="B10" s="3" t="inlineStr">
         <is>
           <t># A grief-focused web app — design exploration
-**Situation.** We're scoping a web product for people in active grief. The space today splits roughly three ways: funeral logistics sites (transactional, mostly pre-funeral), peer support communities and subreddits (exposing or noisy for many), and journaling apps that bolt on a "feeling sad" mood tag (toothless). The users we keep hearing from describe wanting something different — something that respects them as someone grieving rather than treating them as a user to be moved through a funnel or a feed.
-**Complication.** People reach for a tool at the awkward moments: 3am, the anniversary, after a hard conversation with a sibling about settling the estate, on a Tuesday for no specific reason. At those moments, the funeral sites read transactional, the subreddits feel either welcoming or hostile depending on luck, and the mood-tag prompt asks "how are you feeling today?" as if grief were a state to log. Existing tools fail them by being too prescriptive ("step 4 of 7: write a letter to your loved one") or too generic.
-**Users.** Anyone weeks-to-months out from a meaningful loss — recent enough that grief is shaping the day, not so recent that they're still in funeral logistics. The losses vary: parent, partner, friend, pregnancy, pet, anticipatory loss with a terminal diagnosis. The support systems around them vary more — some surrounded by attentive friends, others whose network has gone quiet at six weeks.
-**Cost.** The cost of failure isn't dramatic — it's the slow drift away from a tool that doesn't meet them, and the continued absence of a place that does. What we want from this round: distinct strategic directions for what "a web app for grief" could meaningfully be — real bets that could move the category, not convergent variants.</t>
+## Situation
+We're scoping a web product for people in active grief. The space today splits roughly three ways: funeral logistics sites (transactional, mostly pre-funeral), peer support communities and subreddits (exposing or noisy for many), and journaling apps that bolt on a "feeling sad" mood tag (toothless). The users we keep hearing from describe wanting something different — something that respects them as someone grieving rather than treating them as a user to be moved through a funnel or a feed.
+## Complication
+People reach for a tool at the awkward moments: 3am, the anniversary, after a hard conversation with a sibling about settling the estate, on a Tuesday for no specific reason. At those moments, the funeral sites read transactional, the subreddits feel either welcoming or hostile depending on luck, and the mood-tag prompt asks "how are you feeling today?" as if grief were a state to log. Existing tools fail them by being too prescriptive ("step 4 of 7: write a letter to your loved one") or too generic.
+## Users
+Anyone weeks-to-months out from a meaningful loss — recent enough that grief is shaping the day, not so recent that they're still in funeral logistics. The losses vary: parent, partner, friend, pregnancy, pet, anticipatory loss with a terminal diagnosis. The support systems around them vary more — some surrounded by attentive friends, others whose network has gone quiet at six weeks.
+## Cost
+The cost of failure isn't dramatic — it's the slow drift away from a tool that doesn't meet them, and the continued absence of a place that does. What we want from this round: distinct strategic directions for what "a web app for grief" could meaningfully be — real bets that could move the category, not convergent variants.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1022,10 +1058,14 @@
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t># Discharge instructions for older adults going home — design exploration
-**Situation.** An older adult is being discharged from the hospital this afternoon after a heart-failure exacerbation, a stroke, a fall, or pneumonia. A family caregiver — often an adult child who has travelled in — will run the first week or two at home. The nurse has roughly fifteen minutes to walk through six pages of paperwork before the next admission needs the room.
-**Complication.** The patient is in pain, on medications that affect cognition, exhausted and emotionally activated; what they remember of those fifteen minutes once home is fragmentary. The caregiver who will administer the next thirty days is sometimes in the room and sometimes not. A few days later, the patient is trying to figure out which white pill is the new beta-blocker, what "weigh yourself daily and call if you gain more than three pounds in a week" means in practice, whether today's ankle swelling is a warning sign, and what the printed phone number is for after hours. The discharge papers are face-down on the kitchen table next to the medication bottles. The follow-up is in eleven days.
-**Users.** The dyad post-discharge: the older adult patient recovering at home, and the family caregiver — often an adult child — running the first week or two of medications, warning signs, and follow-up logistics. The discharging nurse and follow-up clinic are stakeholders the design accommodates; the design is for the dyad once paperwork has come home.
-**Cost.** Between now and the follow-up, it is the patient and the caregiver and the paperwork. The cost of getting it wrong is a missed warning sign, a doubled medication, a readmission. Scope is the discharge moment plus the first 7–14 days at home; the clinical care plan is out of scope.</t>
+## Situation
+An older adult is being discharged from the hospital this afternoon after a heart-failure exacerbation, a stroke, a fall, or pneumonia. A family caregiver — often an adult child who has travelled in — will run the first week or two at home. The nurse has roughly fifteen minutes to walk through six pages of paperwork before the next admission needs the room.
+## Complication
+The patient is in pain, on medications that affect cognition, exhausted and emotionally activated; what they remember of those fifteen minutes once home is fragmentary. The caregiver who will administer the next thirty days is sometimes in the room and sometimes not. A few days later, the patient is trying to figure out which white pill is the new beta-blocker, what "weigh yourself daily and call if you gain more than three pounds in a week" means in practice, whether today's ankle swelling is a warning sign, and what the printed phone number is for after hours. The discharge papers are face-down on the kitchen table next to the medication bottles. The follow-up is in eleven days.
+## Users
+The dyad post-discharge: the older adult patient recovering at home, and the family caregiver — often an adult child — running the first week or two of medications, warning signs, and follow-up logistics. The discharging nurse and follow-up clinic are stakeholders the design accommodates; the design is for the dyad once paperwork has come home.
+## Cost
+Between now and the follow-up, it is the patient and the caregiver and the paperwork. The cost of getting it wrong is a missed warning sign, a doubled medication, a readmission. Scope is the discharge moment plus the first 7–14 days at home; the clinical care plan is out of scope.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1082,10 +1122,14 @@
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t># Self-representation in housing court — design exploration
-**Situation.** A tenant has received an eviction notice. Their landlord has filed in housing court. They have a court date in two to three weeks. They cannot afford an attorney; the legal-aid clinic in their county is at capacity. The available self-help resources are accurate, thorough, and unusable in their situation: long PDFs of legalese for someone who is working two jobs and putting kids to bed at the same time.
-**Complication.** The tenant may or may not have a legal defense. The landlord may not have given proper notice; the rent claim may be wrong; the unit may be uninhabitable; the landlord may have engaged in unlawful self-help. Or the tenant may not have a defense and needs to negotiate time, settle, or simply file an answer to preserve options. They have a stack of papers in three different formats, a phone, and an internet connection. They cannot tell which of the eighty pieces of available advice apply to their facts and which don't.
-**Users.** A pro-se tenant facing an eviction filing with a court date two to three weeks out, navigating the case alone. Legal-aid attorneys, court clerks, and the landlord's counsel are stakeholders the tenant encounters; the design is for the tenant doing the work between notice and hearing.
-**Cost.** What they need is to walk into court understanding what is about to happen and what they should say. The cost of falling short is a default judgment, a lost home, and a record that follows them to the next lease application. The scope is from "I got a notice" through "I have prepared for court."</t>
+## Situation
+A tenant has received an eviction notice. Their landlord has filed in housing court. They have a court date in two to three weeks. They cannot afford an attorney; the legal-aid clinic in their county is at capacity. The available self-help resources are accurate, thorough, and unusable in their situation: long PDFs of legalese for someone who is working two jobs and putting kids to bed at the same time.
+## Complication
+The tenant may or may not have a legal defense. The landlord may not have given proper notice; the rent claim may be wrong; the unit may be uninhabitable; the landlord may have engaged in unlawful self-help. Or the tenant may not have a defense and needs to negotiate time, settle, or simply file an answer to preserve options. They have a stack of papers in three different formats, a phone, and an internet connection. They cannot tell which of the eighty pieces of available advice apply to their facts and which don't.
+## Users
+A pro-se tenant facing an eviction filing with a court date two to three weeks out, navigating the case alone. Legal-aid attorneys, court clerks, and the landlord's counsel are stakeholders the tenant encounters; the design is for the tenant doing the work between notice and hearing.
+## Cost
+What they need is to walk into court understanding what is about to happen and what they should say. The cost of falling short is a default judgment, a lost home, and a record that follows them to the next lease application. The scope is from "I got a notice" through "I have prepared for court."</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1140,10 +1184,14 @@
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t># Multi-currency expense report submission — design exploration
-**Situation.** A traveler is home for two days between business trips. The trip that just ended ran through three countries, with receipts in five formats, photos of meals in a foreign language, an airline charge that hit their card in USD but was billed in EUR, a hotel charge pre-authorized at one amount and posted at another, an Uber auto-uploaded but mis-categorized as personal, and a cash tip paid because the card terminal was broken. They have policy questions — was the upgraded flight reimbursable, what counts as a client meal — and no one to ask quickly.
-**Complication.** They submit. Finance rejects it for a single category mismatch and asks them to redo. Each round of back-and-forth is another evening they don't have. The available expense tools present categorization screens, FX-rate prompts, and approval flows; the gap between what the traveler can produce on a Saturday afternoon and what finance needs to approve is where the loop lives.
-**Users.** The business traveler reconciling between trips — competent, time-starved, working from a kitchen table with a phone full of receipts. The finance reviewer reads what was submitted and often sends it back; they are a stakeholder, not the target.
-**Cost.** Evenings lost to resubmissions, the next trip approaching with last trip's report still open, reimbursements that lag for weeks, and the slow erosion of any sense that this part of the job is tractable. The traveler is leaving for São Paulo on Sunday. The scope is from the moment a trip ends to the moment the report is approved.</t>
+## Situation
+A traveler is home for two days between business trips. The trip that just ended ran through three countries, with receipts in five formats, photos of meals in a foreign language, an airline charge that hit their card in USD but was billed in EUR, a hotel charge pre-authorized at one amount and posted at another, an Uber auto-uploaded but mis-categorized as personal, and a cash tip paid because the card terminal was broken. They have policy questions — was the upgraded flight reimbursable, what counts as a client meal — and no one to ask quickly.
+## Complication
+They submit. Finance rejects it for a single category mismatch and asks them to redo. Each round of back-and-forth is another evening they don't have. The available expense tools present categorization screens, FX-rate prompts, and approval flows; the gap between what the traveler can produce on a Saturday afternoon and what finance needs to approve is where the loop lives.
+## Users
+The business traveler reconciling between trips — competent, time-starved, working from a kitchen table with a phone full of receipts. The finance reviewer reads what was submitted and often sends it back; they are a stakeholder, not the target.
+## Cost
+Evenings lost to resubmissions, the next trip approaching with last trip's report still open, reimbursements that lag for weeks, and the slow erosion of any sense that this part of the job is tractable. The traveler is leaving for São Paulo on Sunday. The scope is from the moment a trip ends to the moment the report is approved.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1199,10 +1247,14 @@
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t># A parent finding tutoring for a child struggling in math — design exploration
-**Situation.** A child in 4th, 6th, or 8th grade is struggling in math. The grades have slipped; the teacher has sent a note; the standardized test result came back lower than expected. The parent has a few hours over the next two weeks to set something up, working evenings around their own job and the rest of the family's calendar.
-**Complication.** The parent is facing a tangle of options the landscape currently presents: the local tutoring chain (predictable but expensive, small-group, weekly); a private tutor matched through a friend (variable quality and availability); online tutoring marketplaces and free practice platforms; the school's own intervention program if the kid qualifies; AI-tutor apps that promise personalization. The parent cannot easily tell which option is matched to what works versus what's marketing. They are not the math expert.
-**Users.** A parent–child dyad at the moment of choosing help. The parent is the procurer and decider — scheduling, paying, reading reviews, judging fit. The child is the recipient and the one whose engagement determines whether any of this works; they are sensitive to the framing, since *you need a tutor* can feel like a judgment, and a kid who closes off doesn't learn from anyone. Tutor candidates and school staff are stakeholders the design accommodates, not the target.
-**Cost.** Weeks pass while the parent stalls between bad options; the child falls further behind in a subject that compounds; the wrong choice burns money and the child's willingness to try again. The scope is from "we need help" through "we have a plan and a tutor we trust."</t>
+## Situation
+A child in 4th, 6th, or 8th grade is struggling in math. The grades have slipped; the teacher has sent a note; the standardized test result came back lower than expected. The parent has a few hours over the next two weeks to set something up, working evenings around their own job and the rest of the family's calendar.
+## Complication
+The parent is facing a tangle of options the landscape currently presents: the local tutoring chain (predictable but expensive, small-group, weekly); a private tutor matched through a friend (variable quality and availability); online tutoring marketplaces and free practice platforms; the school's own intervention program if the kid qualifies; AI-tutor apps that promise personalization. The parent cannot easily tell which option is matched to what works versus what's marketing. They are not the math expert.
+## Users
+A parent–child dyad at the moment of choosing help. The parent is the procurer and decider — scheduling, paying, reading reviews, judging fit. The child is the recipient and the one whose engagement determines whether any of this works; they are sensitive to the framing, since *you need a tutor* can feel like a judgment, and a kid who closes off doesn't learn from anyone. Tutor candidates and school staff are stakeholders the design accommodates, not the target.
+## Cost
+Weeks pass while the parent stalls between bad options; the child falls further behind in a subject that compounds; the wrong choice burns money and the child's willingness to try again. The scope is from "we need help" through "we have a plan and a tutor we trust."</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1257,10 +1309,14 @@
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t># Pre-travel prescription preparation — design exploration
-**Situation.** A person is preparing for a long international trip. They take regular prescription medication — an SSRI, an ADHD stimulant, a blood thinner, hormone therapy, a controlled-substance painkiller. They are two weeks out and just realized this is harder than they thought. US prescriptions can't be filled at overseas pharmacies. Several common US medications are restricted or illegal in the country they're going to.
-**Complication.** To carry enough for the trip, they need a vacation override from their insurance, weeks in advance, and probably a prescriber letter. None of that is one phone call. They are working it out across pharmacy phone trees, the insurer's app, the State Department's site, and Reddit threads. Their PCP's office is not set up to answer travel-medication questions. The pharmacy can fill the script if the doctor authorizes the override; the doctor will authorize the override if asked correctly. Nobody owns the work of getting this person across the world with their medication intact, legal, and packaged the way customs expects.
-**Users.** An international traveler on regular, often controlled, prescription medication — a person managing real conditions who needs to keep managing them on the other side of a border. Prescriber, pharmacist, insurer, and customs are stakeholders this work moves through, not the target.
-**Cost.** Consequences run from confiscation at customs to denial of entry to arrest in stricter jurisdictions, plus the quieter failure of running out of medication mid-trip and the destabilization that follows. The scope is the four-week window before international departure.</t>
+## Situation
+A person is preparing for a long international trip. They take regular prescription medication — an SSRI, an ADHD stimulant, a blood thinner, hormone therapy, a controlled-substance painkiller. They are two weeks out and just realized this is harder than they thought. US prescriptions can't be filled at overseas pharmacies. Several common US medications are restricted or illegal in the country they're going to.
+## Complication
+To carry enough for the trip, they need a vacation override from their insurance, weeks in advance, and probably a prescriber letter. None of that is one phone call. They are working it out across pharmacy phone trees, the insurer's app, the State Department's site, and Reddit threads. Their PCP's office is not set up to answer travel-medication questions. The pharmacy can fill the script if the doctor authorizes the override; the doctor will authorize the override if asked correctly. Nobody owns the work of getting this person across the world with their medication intact, legal, and packaged the way customs expects.
+## Users
+An international traveler on regular, often controlled, prescription medication — a person managing real conditions who needs to keep managing them on the other side of a border. Prescriber, pharmacist, insurer, and customs are stakeholders this work moves through, not the target.
+## Cost
+Consequences run from confiscation at customs to denial of entry to arrest in stricter jurisdictions, plus the quieter failure of running out of medication mid-trip and the destabilization that follows. The scope is the four-week window before international departure.</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1300,10 +1356,14 @@
       <c r="B16" s="3" t="inlineStr">
         <is>
           <t># Finding a primary care doctor after relocating — design exploration
-**Situation.** A person has moved to a new city and needs a primary care doctor. They have insurance, and their plan's website hands them an in-network directory — several hundred names, sorted by ZIP code. The directory shows specialties and addresses. It rarely shows which practices are accepting new patients, what the next available appointment actually is, which clinicians speak the languages spoken in the patient's household, whether the office is wheelchair-accessible, or how the practice handles diabetes care, mental-health needs, or pregnancy.
-**Complication.** The patient calls one office, sits on hold for ten minutes, navigates a phone tree, and is told the next opening is in five months — or that the practice isn't accepting new patients at all. Then the next call. Then the next. The options they are choosing between in the landscape today include the in-network directory itself, telehealth services their plan covers, federally-qualified health centers in the area, and direct primary care practices that bill outside insurance — none of which the directory surfaces side-by-side.
-**Users.** A patient looking for a primary care doctor in a new city. Some have active conditions — chronic pain, diabetes, anxiety — and need to start care now; others are establishing routine care and re-engage only when something goes wrong. The insurance plan, the in-network directory, the practices, and telehealth providers are stakeholder context the design accommodates, not the target.
-**Cost.** Delayed care for people who need it now; undiagnosed conditions for those who give up early; emergency visits for what should have been clinic visits. The scope is from "I need a new doctor" through "I have an appointment booked."</t>
+## Situation
+A person has moved to a new city and needs a primary care doctor. They have insurance, and their plan's website hands them an in-network directory — several hundred names, sorted by ZIP code. The directory shows specialties and addresses. It rarely shows which practices are accepting new patients, what the next available appointment actually is, which clinicians speak the languages spoken in the patient's household, whether the office is wheelchair-accessible, or how the practice handles diabetes care, mental-health needs, or pregnancy.
+## Complication
+The patient calls one office, sits on hold for ten minutes, navigates a phone tree, and is told the next opening is in five months — or that the practice isn't accepting new patients at all. Then the next call. Then the next. The options they are choosing between in the landscape today include the in-network directory itself, telehealth services their plan covers, federally-qualified health centers in the area, and direct primary care practices that bill outside insurance — none of which the directory surfaces side-by-side.
+## Users
+A patient looking for a primary care doctor in a new city. Some have active conditions — chronic pain, diabetes, anxiety — and need to start care now; others are establishing routine care and re-engage only when something goes wrong. The insurance plan, the in-network directory, the practices, and telehealth providers are stakeholder context the design accommodates, not the target.
+## Cost
+Delayed care for people who need it now; undiagnosed conditions for those who give up early; emergency visits for what should have been clinic visits. The scope is from "I need a new doctor" through "I have an appointment booked."</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1344,10 +1404,14 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t># Remote new-hire onboarding, week one — design exploration
-**Situation.** A competent professional joins a remote-first company on Monday. They have never met their team in person. They've done this before — they know how to set up a laptop and learn a new codebase. The HR-built first week is nine meetings Monday, six Tuesday; a stack of documentation; a Notion they still can't fully access; benefits links, security trainings, and a Slack workspace with a hundred channels.
-**Complication.** What's hard isn't the work; it's everything around it. They don't know this team's norms, this manager's actual (not stated) preferences, who is the person you actually ask about benefits. Remote replaces the watercooler, the lunch tag-along, and the overheard standup with calendar invites — which aren't the same thing. By Wednesday the orientation rush slows; by Thursday they're alone with documentation and unsure who to ask what, anxious about asking questions that would mark them as not-yet-onboard.
-**Users.** The new hire — a competent professional starting cold inside a remote-first company, navigating their first five working days from a home desk. The hiring manager, peers on the team, HR, and IT provisioning are stakeholders whose work shapes the week but who are not the target of the design.
-**Cost.** The five-day window from joining to belonging is where the relationship is made or lost; new hires who don't feel onboard by Friday carry that uncertainty into the next month, hesitate to ask, and quietly disengage. Companies bleed early-tenure hires at exactly this point. The scope is the first five working days, Monday morning to Friday afternoon.</t>
+## Situation
+A competent professional joins a remote-first company on Monday. They have never met their team in person. They've done this before — they know how to set up a laptop and learn a new codebase. The HR-built first week is nine meetings Monday, six Tuesday; a stack of documentation; a Notion they still can't fully access; benefits links, security trainings, and a Slack workspace with a hundred channels.
+## Complication
+What's hard isn't the work; it's everything around it. They don't know this team's norms, this manager's actual (not stated) preferences, who is the person you actually ask about benefits. Remote replaces the watercooler, the lunch tag-along, and the overheard standup with calendar invites — which aren't the same thing. By Wednesday the orientation rush slows; by Thursday they're alone with documentation and unsure who to ask what, anxious about asking questions that would mark them as not-yet-onboard.
+## Users
+The new hire — a competent professional starting cold inside a remote-first company, navigating their first five working days from a home desk. The hiring manager, peers on the team, HR, and IT provisioning are stakeholders whose work shapes the week but who are not the target of the design.
+## Cost
+The five-day window from joining to belonging is where the relationship is made or lost; new hires who don't feel onboard by Friday carry that uncertainty into the next month, hesitate to ask, and quietly disengage. Companies bleed early-tenure hires at exactly this point. The scope is the first five working days, Monday morning to Friday afternoon.</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1402,10 +1466,14 @@
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t># A sprint retro after a missed target — design exploration
-**Situation.** A product team has just finished a two-week sprint and missed what they committed to. The scrum master has forty-five minutes booked on Friday afternoon for the retrospective. The team is tired, the engineer who carried the cancelled feature is quiet on the call, the PM is reading their phone, and the VP of Engineering is on the line listening in. The scrum master has a Miro board with three columns and a stack of sticky notes their team has used in some version for the last two years.
-**Complication.** The team's existing tools — Miro templates, FunRetro, EasyRetro, the Jira retro module — capture sticky notes and let people upvote them. What happens between "sticky notes captured" and "the team had a real conversation" sits outside those tools. The team itself is uneven: some members will say what they think directly, some won't say anything that could read as criticism with the PM in the room, and some will narrate the sprint as if it went fine.
-**Users.** The scrum master is the target user — the one prepping the meeting, holding the room, and chasing follow-through. The team is the design's audience; the PM in the room and the VP listening in are stakeholders the meeting accommodates.
-**Cost.** A retro that doesn't land after a missed sprint compounds: the same patterns carry into the next sprint, action items are forgotten by Monday, and the team grows a little more cynical about whether retros are worth showing up to. A retro that does land is something the team can feel for weeks. The scope is the retrospective meeting itself, the prep before it, and the follow-through.</t>
+## Situation
+A product team has just finished a two-week sprint and missed what they committed to. The scrum master has forty-five minutes booked on Friday afternoon for the retrospective. The team is tired, the engineer who carried the cancelled feature is quiet on the call, the PM is reading their phone, and the VP of Engineering is on the line listening in. The scrum master has a Miro board with three columns and a stack of sticky notes their team has used in some version for the last two years.
+## Complication
+The team's existing tools — Miro templates, FunRetro, EasyRetro, the Jira retro module — capture sticky notes and let people upvote them. What happens between "sticky notes captured" and "the team had a real conversation" sits outside those tools. The team itself is uneven: some members will say what they think directly, some won't say anything that could read as criticism with the PM in the room, and some will narrate the sprint as if it went fine.
+## Users
+The scrum master is the target user — the one prepping the meeting, holding the room, and chasing follow-through. The team is the design's audience; the PM in the room and the VP listening in are stakeholders the meeting accommodates.
+## Cost
+A retro that doesn't land after a missed sprint compounds: the same patterns carry into the next sprint, action items are forgotten by Monday, and the team grows a little more cynical about whether retros are worth showing up to. A retro that does land is something the team can feel for weeks. The scope is the retrospective meeting itself, the prep before it, and the follow-through.</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1446,10 +1514,14 @@
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t># Applying for food assistance — design exploration
-**Situation.** Someone who needs food assistance now is sitting down to apply for SNAP. They've lost a job, had hours cut, gotten sick, or are raising a kid on inconsistent income. They are working from a phone, sometimes a shared one, often on intermittent data.
-**Complication.** The form in front of them asks branching questions whose answers depend on context the form does not let them explain, requires documents they can't easily produce in the moment (a recent pay stub from a gig that pays inconsistently, a lease they don't have a copy of, a Social Security card from a drawer at a place they no longer live), and was built to be filled out on a desktop computer they don't own. After they submit, the experience goes quiet. They don't know if the application was received, is being processed, is waiting on a document the system has not asked for, or has already been denied.
-**Users.** The target user is the applicant: a first-time applicant who has never used the safety net, a mixed-status family weighing whether the application itself will be used against them, or someone returning under worse circumstances than the first time. State eligibility workers who process and adjudicate these applications are stakeholders, not the target.
-**Cost.** Days pass. The food situation that brought them here doesn't pause. Many people in this position get one attempt before they stop trying — not from a single rejection, but from the cumulative weight of submitting into silence while the rest of their life keeps moving. What we want: distinct strategic directions for what a humane food-assistance application could be when designed around the applicant.</t>
+## Situation
+Someone who needs food assistance now is sitting down to apply for SNAP. They've lost a job, had hours cut, gotten sick, or are raising a kid on inconsistent income. They are working from a phone, sometimes a shared one, often on intermittent data.
+## Complication
+The form in front of them asks branching questions whose answers depend on context the form does not let them explain, requires documents they can't easily produce in the moment (a recent pay stub from a gig that pays inconsistently, a lease they don't have a copy of, a Social Security card from a drawer at a place they no longer live), and was built to be filled out on a desktop computer they don't own. After they submit, the experience goes quiet. They don't know if the application was received, is being processed, is waiting on a document the system has not asked for, or has already been denied.
+## Users
+The target user is the applicant: a first-time applicant who has never used the safety net, a mixed-status family weighing whether the application itself will be used against them, or someone returning under worse circumstances than the first time. State eligibility workers who process and adjudicate these applications are stakeholders, not the target.
+## Cost
+Days pass. The food situation that brought them here doesn't pause. Many people in this position get one attempt before they stop trying — not from a single rejection, but from the cumulative weight of submitting into silence while the rest of their life keeps moving. What we want: distinct strategic directions for what a humane food-assistance application could be when designed around the applicant.</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1504,10 +1576,14 @@
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t># The first 90 days after a Type 2 diabetes diagnosis — design exploration
-**Situation.** A person has just been told they have Type 2 diabetes. The diagnosis arrived in a fifteen-minute appointment with a handout, a prescription for metformin, and instructions to "watch your sugars" and to "see a nutritionist." They walk out scared, ashamed, confused about whether they caused this, and facing a slate of changes — diet, exercise, medication, glucose monitoring, A1c labs every three months.
-**Complication.** No one helps them sequence those changes. The nutritionist referral is a phone number on the printout. The diabetes self-management education and support sessions their insurance covers are not mentioned at the appointment. The landscape they encounter when they look for help — glucose-logging utilities, coaching platforms (Livongo, Virta, Omada), peer-support communities, and YouTube videos from creators of varying authority — tends to ask them to log their glucose on day one. None of it is shaped around the moment of diagnosis itself: the week they are still telling family, the week they are deciding whether to tell work.
-**Users.** The target user is the newly-diagnosed patient in the first 90 days. The clinician and the nutritionist are stakeholders the design accommodates — referrals come from them, labs route through them — but are not who the design is for.
-**Cost.** By the end of the next ninety days they will have either built a workable rhythm — meals, walking, the morning metformin, the glucose meter sitting on the kitchen counter — or they will have drifted: meter in a drawer, prescription unfilled at refill time, weight unchanged, and no further appointment booked until the next labs flag something. The scope is from diagnosis through the 90-day mark.</t>
+## Situation
+A person has just been told they have Type 2 diabetes. The diagnosis arrived in a fifteen-minute appointment with a handout, a prescription for metformin, and instructions to "watch your sugars" and to "see a nutritionist." They walk out scared, ashamed, confused about whether they caused this, and facing a slate of changes — diet, exercise, medication, glucose monitoring, A1c labs every three months.
+## Complication
+No one helps them sequence those changes. The nutritionist referral is a phone number on the printout. The diabetes self-management education and support sessions their insurance covers are not mentioned at the appointment. The landscape they encounter when they look for help — glucose-logging utilities, coaching platforms (Livongo, Virta, Omada), peer-support communities, and YouTube videos from creators of varying authority — tends to ask them to log their glucose on day one. None of it is shaped around the moment of diagnosis itself: the week they are still telling family, the week they are deciding whether to tell work.
+## Users
+The target user is the newly-diagnosed patient in the first 90 days. The clinician and the nutritionist are stakeholders the design accommodates — referrals come from them, labs route through them — but are not who the design is for.
+## Cost
+By the end of the next ninety days they will have either built a workable rhythm — meals, walking, the morning metformin, the glucose meter sitting on the kitchen counter — or they will have drifted: meter in a drawer, prescription unfilled at refill time, weight unchanged, and no further appointment booked until the next labs flag something. The scope is from diagnosis through the 90-day mark.</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1547,10 +1623,14 @@
       <c r="B21" s="3" t="inlineStr">
         <is>
           <t># Filing for unemployment insurance — design exploration
-**Situation.** A person has just lost their job and is filing for unemployment insurance through their state's labor agency. They may have a few weeks of rent in the bank or none. They are filling out the application on a phone — in line at a job center, between caregiving shifts, or late at night after the kids are asleep.
-**Complication.** The application asks for an EDDCAN number they have never heard of, pay stubs from the last eighteen months they may not have saved, and the precise dates and hours of every job worked in a base period that doesn't match how variable-schedule work happens. The legalese is dense. A wrong answer on any of dozens of questions delays or denies the claim, and the appeal that follows takes weeks. Once filed, the channels for finding out what's happening are a state portal that often shows information weeks out of date, paper letters that arrive after the next pay period would have been due, and a phone line that holds for hours. The portal sometimes says the claim is being processed; sometimes nothing at all.
-**Users.** The target user is the claimant — filing and waiting on benefits they are entitled to under state and federal law. State eligibility workers and adjudicators are stakeholders, not the target.
-**Cost.** Money does not arrive on a schedule the person can plan around. Rent is due, the car insurance lapses, the kid needs school supplies. The gap between filing and the first payment landing is where the urgency of the situation collides with what the system communicates. The scope is the filing flow plus the first thirty days of claim-status communication.</t>
+## Situation
+A person has just lost their job and is filing for unemployment insurance through their state's labor agency. They may have a few weeks of rent in the bank or none. They are filling out the application on a phone — in line at a job center, between caregiving shifts, or late at night after the kids are asleep.
+## Complication
+The application asks for an EDDCAN number they have never heard of, pay stubs from the last eighteen months they may not have saved, and the precise dates and hours of every job worked in a base period that doesn't match how variable-schedule work happens. The legalese is dense. A wrong answer on any of dozens of questions delays or denies the claim, and the appeal that follows takes weeks. Once filed, the channels for finding out what's happening are a state portal that often shows information weeks out of date, paper letters that arrive after the next pay period would have been due, and a phone line that holds for hours. The portal sometimes says the claim is being processed; sometimes nothing at all.
+## Users
+The target user is the claimant — filing and waiting on benefits they are entitled to under state and federal law. State eligibility workers and adjudicators are stakeholders, not the target.
+## Cost
+Money does not arrive on a schedule the person can plan around. Rent is due, the car insurance lapses, the kid needs school supplies. The gap between filing and the first payment landing is where the urgency of the situation collides with what the system communicates. The scope is the filing flow plus the first thirty days of claim-status communication.</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1590,10 +1670,14 @@
       <c r="B22" s="3" t="inlineStr">
         <is>
           <t># Updating voter registration after a name change — design exploration
-**Situation.** A person has changed their legal name — after marriage, divorce, gender transition, leaving an abusive relationship, or by personal choice. Their old name is on the voter roll. The next election is months away. Someone told them they should update their registration; they don't know whether they need to, by when, what proof, or how their state's rules differ from a friend's in another state.
-**Complication.** The state election-board website is a tangle of pages and PDFs that don't quite match their situation. Voter registration sits inside a long list of bureaucratic to-dos the name change has triggered — driver's license, Social Security card, employer records, banking, passports — and is the one most likely to be skipped until election day.
-**Users.** The target user is the voter mid-name-change: a trans person whose ID is finally catching up to their name, a domestic-violence survivor who changed their name for safety, a recently-married or recently-divorced voter, or someone who chose a new name. Each comes with different proof, different timelines, and different concerns about who sees the old name during the update. Election-board staff and poll workers are stakeholders, not the target.
-**Cost.** On election day, the name fails the poll-book check and they're asked to cast a provisional ballot they may not return to cure. A vote they were entitled to cast doesn't count, and being challenged at the table — especially for trans voters or survivors whose old name is read aloud — can make them less likely to return. The scope is updating registration plus the ambiguity around it — *do I need to, when by, what proof, will this be wrong on election day.*</t>
+## Situation
+A person has changed their legal name — after marriage, divorce, gender transition, leaving an abusive relationship, or by personal choice. Their old name is on the voter roll. The next election is months away. Someone told them they should update their registration; they don't know whether they need to, by when, what proof, or how their state's rules differ from a friend's in another state.
+## Complication
+The state election-board website is a tangle of pages and PDFs that don't quite match their situation. Voter registration sits inside a long list of bureaucratic to-dos the name change has triggered — driver's license, Social Security card, employer records, banking, passports — and is the one most likely to be skipped until election day.
+## Users
+The target user is the voter mid-name-change: a trans person whose ID is finally catching up to their name, a domestic-violence survivor who changed their name for safety, a recently-married or recently-divorced voter, or someone who chose a new name. Each comes with different proof, different timelines, and different concerns about who sees the old name during the update. Election-board staff and poll workers are stakeholders, not the target.
+## Cost
+On election day, the name fails the poll-book check and they're asked to cast a provisional ballot they may not return to cure. A vote they were entitled to cast doesn't count, and being challenged at the table — especially for trans voters or survivors whose old name is read aloud — can make them less likely to return. The scope is updating registration plus the ambiguity around it — *do I need to, when by, what proof, will this be wrong on election day.*</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
refactor(briefs): revert SCUC headers from H2 to inline-bold labels
The H2 block-heading format (`## Situation` on its own line) invoked
heading-level rendering in the canvas brief node, treating the SCUC
slots as a sectioned document rather than a four-paragraph problem
statement. Revert to inline-bold labels (`**Situation.** Text…`) so
SCUC labels are visible in the prompt as text emphasis only — no
special block treatment from the node, brief reads as prose.

Skill section 1.3 reverted to teach the inline-bold form as canonical.
corpus-content.xlsx refreshed.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/corpus-content.xlsx
+++ b/experiments/corpus-content.xlsx
@@ -503,14 +503,10 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t># Apartment search for a renter with a past eviction — design exploration
-## Situation
-A person with an eviction record is looking for a new place to live. The eviction may have followed a job loss, a medical event, or a dispute with a prior landlord — sometimes a dismissed filing, sometimes a filing-in-error, sometimes a completed eviction-for-cause. The renter has since rebuilt: a job, references, money for a deposit. What reaches the landlord is a tenant-screening report — bundling rental, credit, employment, and criminal history into a score — on which the filing looks the same whether the case was won, lost, or dismissed.
-## Complication
-The renter pays application fees at every listing and discovers, sometimes days later, that they have been declined. They get back a vague "did not meet screening criteria" or no explanation at all. There is no path to find out which factor produced the decline, no path to contest a record they believe is inaccurate. They confront listing aggregators, screening companies whose reports they cannot see, bureau disputes that move slowly, and legal-aid offices whose capacity does not meet the volume.
-## Users
-The renter with the eviction record on their file. Landlords and screening companies are stakeholders, not the target — the design is for the renter with weeks, not months, and a stack of declined applications. Scope is "I'm looking" through "I've signed a lease."
-## Cost
-They need to be housed in the weeks they have, not the months a dispute would take. Fees stack up against a deposit they are trying to keep intact. Each decline arrives without enough information to act on, and the next listing goes up against the same report. The current housing is running out or already gone.</t>
+**Situation.** A person with an eviction record is looking for a new place to live. The eviction may have followed a job loss, a medical event, or a dispute with a prior landlord — sometimes a dismissed filing, sometimes a filing-in-error, sometimes a completed eviction-for-cause. The renter has since rebuilt: a job, references, money for a deposit. What reaches the landlord is a tenant-screening report — bundling rental, credit, employment, and criminal history into a score — on which the filing looks the same whether the case was won, lost, or dismissed.
+**Complication.** The renter pays application fees at every listing and discovers, sometimes days later, that they have been declined. They get back a vague "did not meet screening criteria" or no explanation at all. There is no path to find out which factor produced the decline, no path to contest a record they believe is inaccurate. They confront listing aggregators, screening companies whose reports they cannot see, bureau disputes that move slowly, and legal-aid offices whose capacity does not meet the volume.
+**Users.** The renter with the eviction record on their file. Landlords and screening companies are stakeholders, not the target — the design is for the renter with weeks, not months, and a stack of declined applications. Scope is "I'm looking" through "I've signed a lease."
+**Cost.** They need to be housed in the weeks they have, not the months a dispute would take. Fees stack up against a deposit they are trying to keep intact. Each decline arrives without enough information to act on, and the next listing goes up against the same report. The current housing is running out or already gone.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -566,14 +562,10 @@
       <c r="B3" s="3" t="inlineStr">
         <is>
           <t># Coordinating care for an aging parent — design exploration
-## Situation
-An adult child is responsible for the day-to-day care of an aging parent in another city. They are working full-time, may be raising their own kids, and are now also managing their parent's medications, appointments, insurance disputes, in-home aide schedule, finances, and longer-term decisions about home modifications, assisted living, or hospice — with sibling involvement that ranges from supportive to fractious.
-## Complication
-The information lives everywhere — their own phone, their email, the parent's hand-written notes on a yellow pad by the kitchen phone, the parent's doctor's portals (three or four, each with its own login), Medicare statements, the aide's notebook, the pharmacy's text messages. No system holds the picture; the caregiver holds it, in their head, between work meetings and bedtime. The new prescription started last Thursday is supposed to be checked against the cardiologist's older one that may or may not have been discontinued. The PCP's portal does not show the cardiologist's prescriptions. The aide's notebook is three hundred miles away.
-## Users
-The adult-child caregiver and the aging parent, as a dyad — the parent in their own apartment, the caregiver coordinating from three hundred miles away. Siblings, aides, doctors, and pharmacists are stakeholders the design accommodates, not optimizes for. Scope is the rhythm of a month, not a single appointment.
-## Cost
-When something goes wrong — a missed medication, a duplicate dose, an ED visit that looks preventable in hindsight — the gap was between systems the caregiver was supposed to bridge across. The parent absorbs the errors when the picture slips. The work eats evenings, weekends, and the bandwidth left for everything else in the caregiver's life.</t>
+**Situation.** An adult child is responsible for the day-to-day care of an aging parent in another city. They are working full-time, may be raising their own kids, and are now also managing their parent's medications, appointments, insurance disputes, in-home aide schedule, finances, and longer-term decisions about home modifications, assisted living, or hospice — with sibling involvement that ranges from supportive to fractious.
+**Complication.** The information lives everywhere — their own phone, their email, the parent's hand-written notes on a yellow pad by the kitchen phone, the parent's doctor's portals (three or four, each with its own login), Medicare statements, the aide's notebook, the pharmacy's text messages. No system holds the picture; the caregiver holds it, in their head, between work meetings and bedtime. The new prescription started last Thursday is supposed to be checked against the cardiologist's older one that may or may not have been discontinued. The PCP's portal does not show the cardiologist's prescriptions. The aide's notebook is three hundred miles away.
+**Users.** The adult-child caregiver and the aging parent, as a dyad — the parent in their own apartment, the caregiver coordinating from three hundred miles away. Siblings, aides, doctors, and pharmacists are stakeholders the design accommodates, not optimizes for. Scope is the rhythm of a month, not a single appointment.
+**Cost.** When something goes wrong — a missed medication, a duplicate dose, an ED visit that looks preventable in hindsight — the gap was between systems the caregiver was supposed to bridge across. The parent absorbs the errors when the picture slips. The work eats evenings, weekends, and the bandwidth left for everything else in the caregiver's life.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -629,14 +621,10 @@
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t># An adult learner re-entering community college — design exploration
-## Situation
-An adult — twenty-five, thirty-five, fifty — has enrolled at community college, often after years away from formal schooling. They've decided to re-enroll for a new credential, an industry switch, or developmental coursework before a four-year transfer. They've signed up; they haven't started. They have a job that won't easily flex, kids who need pick-up, and the cognitive disjuncture of being asked to think like a student again after years of not being one.
-## Complication
-They are trying to read a college website built for eighteen-year-olds applying for fall. They are unsure where to park, what to bring to orientation, whether the FAFSA they filled out applies to summer term, whether they can register part-time without losing the financial-aid bracket, and how to reach an advisor who answers in less than two weeks.
-## Users
-The adult learner re-entering community college after years away — not the eighteen-year-old applying for fall, and not the returner with a working campus rhythm. Advisors, financial-aid officers, and registrars are stakeholders the design encounters, not optimizes for. Scope is the eight-week window from "I've enrolled" through "I've completed the first month of classes."
-## Cost
-The first month is where the workable rhythm either gets built or doesn't. When the answers don't arrive in the window — when orientation feels alien, when the FAFSA question goes two weeks without a reply, when the parking and pick-up logistics don't line up — the learner quietly stops coming. The enrollment becomes another unfinished credential, the tuition becomes a sunk cost, and the next attempt is years out.</t>
+**Situation.** An adult — twenty-five, thirty-five, fifty — has enrolled at community college, often after years away from formal schooling. They've decided to re-enroll for a new credential, an industry switch, or developmental coursework before a four-year transfer. They've signed up; they haven't started. They have a job that won't easily flex, kids who need pick-up, and the cognitive disjuncture of being asked to think like a student again after years of not being one.
+**Complication.** They are trying to read a college website built for eighteen-year-olds applying for fall. They are unsure where to park, what to bring to orientation, whether the FAFSA they filled out applies to summer term, whether they can register part-time without losing the financial-aid bracket, and how to reach an advisor who answers in less than two weeks.
+**Users.** The adult learner re-entering community college after years away — not the eighteen-year-old applying for fall, and not the returner with a working campus rhythm. Advisors, financial-aid officers, and registrars are stakeholders the design encounters, not optimizes for. Scope is the eight-week window from "I've enrolled" through "I've completed the first month of classes."
+**Cost.** The first month is where the workable rhythm either gets built or doesn't. When the answers don't arrive in the window — when orientation feels alien, when the FAFSA question goes two weeks without a reply, when the parking and pick-up logistics don't line up — the learner quietly stops coming. The enrollment becomes another unfinished credential, the tuition becomes a sunk cost, and the next attempt is years out.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -691,14 +679,10 @@
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t># Disputing a credit-report error — design exploration
-## Situation
-A person has been denied an apartment, a job, a loan, or an insurance rate because of something on their credit report — and the something is wrong. A debt they paid years ago. An account opened in their name fraudulently. Identity confusion with a relative who shares their name. They have proof — receipts, closure letters, identity-theft affidavits — and no clear path to get it to the right place.
-## Complication
-They face three different dispute interfaces, one per bureau, each demanding documentation in slightly different formats and each capable of returning a one-line "investigated, no change" weeks later. They are unsure whether to write a paper letter, use the online portals, file directly with the furnisher, file a CFPB complaint, or do all four. The original error often reappears later from a different furnisher, and the consumer is back at the same three logins, the same documentation queue, the same wait. They confront the bureaus' portals, free-credit-report sites that funnel toward paid monitoring, the CFPB channel, IdentityTheft.gov, and legal-aid whose capacity does not meet the volume.
-## Users
-The consumer disputing the error — the one with receipts and closure letters in hand. Bureaus, furnishers, and CFPB intake staff are stakeholders, not the target. Scope is from noticing the error through resolution.
-## Cost
-The process unfolds over thirty to ninety days while the apartment application sits in limbo and the new job offer is on hold. The denial that prompted the dispute does not pause for resolution. When the error reappears from a different furnisher, the consumer is back at the same three logins, doing the work again on a life that has moved on.</t>
+**Situation.** A person has been denied an apartment, a job, a loan, or an insurance rate because of something on their credit report — and the something is wrong. A debt they paid years ago. An account opened in their name fraudulently. Identity confusion with a relative who shares their name. They have proof — receipts, closure letters, identity-theft affidavits — and no clear path to get it to the right place.
+**Complication.** They face three different dispute interfaces, one per bureau, each demanding documentation in slightly different formats and each capable of returning a one-line "investigated, no change" weeks later. They are unsure whether to write a paper letter, use the online portals, file directly with the furnisher, file a CFPB complaint, or do all four. The original error often reappears later from a different furnisher, and the consumer is back at the same three logins, the same documentation queue, the same wait. They confront the bureaus' portals, free-credit-report sites that funnel toward paid monitoring, the CFPB channel, IdentityTheft.gov, and legal-aid whose capacity does not meet the volume.
+**Users.** The consumer disputing the error — the one with receipts and closure letters in hand. Bureaus, furnishers, and CFPB intake staff are stakeholders, not the target. Scope is from noticing the error through resolution.
+**Cost.** The process unfolds over thirty to ninety days while the apartment application sits in limbo and the new job offer is on hold. The denial that prompted the dispute does not pause for resolution. When the error reappears from a different furnisher, the consumer is back at the same three logins, doing the work again on a life that has moved on.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -753,14 +737,10 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t># First contact with 988, the crisis line — design exploration
-## Situation
-Someone is reaching out to the US crisis line — 988 — for the first time. They may be experiencing a suicidal crisis, an acute panic episode, a substance-use crisis, or distress around grief, abuse, or identity. They may be the person in crisis, or a friend or family member trying to help someone else. They are reaching out at a moment of acute vulnerability and have a choice to make about whether to stay on the line.
-## Complication
-The first sixty seconds are determinative. What does this look like; will I be judged; what's about to happen; will police be sent to my address if I say the wrong thing. People who have heard that police might be dispatched are hesitant in ways the system has to meet; people who have never reached out before are calibrating from the screen, the voice, the hold music. The decision to keep reaching, or to hang up and not try again, is made before anyone has said anything.
-## Users
-The first-time reacher — the person in crisis, or the friend or family member calling on their behalf — in the opening seconds before a counselor has spoken. Counselors and dispatchers are stakeholders the design hands off to, not optimizes for. Scope is the call, text, or chat opening plus the immediate next step; the counselor protocol itself is out of scope.
-## Cost
-When the first sixty seconds don't hold, the person hangs up and does not try again. The next acute moment arrives without a line they trust. The friend who was calling for someone else goes back with nothing to offer.</t>
+**Situation.** Someone is reaching out to the US crisis line — 988 — for the first time. They may be experiencing a suicidal crisis, an acute panic episode, a substance-use crisis, or distress around grief, abuse, or identity. They may be the person in crisis, or a friend or family member trying to help someone else. They are reaching out at a moment of acute vulnerability and have a choice to make about whether to stay on the line.
+**Complication.** The first sixty seconds are determinative. What does this look like; will I be judged; what's about to happen; will police be sent to my address if I say the wrong thing. People who have heard that police might be dispatched are hesitant in ways the system has to meet; people who have never reached out before are calibrating from the screen, the voice, the hold music. The decision to keep reaching, or to hang up and not try again, is made before anyone has said anything.
+**Users.** The first-time reacher — the person in crisis, or the friend or family member calling on their behalf — in the opening seconds before a counselor has spoken. Counselors and dispatchers are stakeholders the design hands off to, not optimizes for. Scope is the call, text, or chat opening plus the immediate next step; the counselor protocol itself is out of scope.
+**Cost.** When the first sixty seconds don't hold, the person hangs up and does not try again. The next acute moment arrives without a line they trust. The friend who was calling for someone else goes back with nothing to offer.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -814,14 +794,10 @@
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t># Closing a deceased family member's accounts — design exploration
-## Situation
-When a person dies, someone in the family inherits an administrative ordeal nobody trained them for. They are the executor — spouse, adult child, sibling — and now need to identify, contact, and close out dozens of accounts: banks, credit cards, utilities, mortgages, retirement accounts, insurance, Social Security, and a digital life of email and photos and subscriptions. They are doing this in the evenings, between the funeral and the rest of life — often from a different city than the deceased, with a death certificate in hand and a stack of unopened mail.
-## Complication
-Each institution has its own forms, its own definitions, its own staff. Debt collectors begin calling within days; most are wrong about what the survivor owes, but the conversations are intimidating and the rules vary by state. The available resources are accurate and encyclopedic; they list eighty things the executor might need to do, with no way to know which twelve apply today.
-## Users
-The executor — spouse, adult child, or sibling — grieving and doing this because someone had to be. Institutions and debt collectors are stakeholders, not the design's target. Scope is from the first week through final dissolution.
-## Cost
-The work runs in the evenings on top of grief, on top of a job, on top of a household that did not pause. The encyclopedic list does not tell the executor which twelve of eighty steps belong to today, so the wrong ones get done first or none at all. The collectors' calls keep coming. The estate stays open, the mail keeps arriving, and the grief is interrupted every time the ordeal reasserts itself.</t>
+**Situation.** When a person dies, someone in the family inherits an administrative ordeal nobody trained them for. They are the executor — spouse, adult child, sibling — and now need to identify, contact, and close out dozens of accounts: banks, credit cards, utilities, mortgages, retirement accounts, insurance, Social Security, and a digital life of email and photos and subscriptions. They are doing this in the evenings, between the funeral and the rest of life — often from a different city than the deceased, with a death certificate in hand and a stack of unopened mail.
+**Complication.** Each institution has its own forms, its own definitions, its own staff. Debt collectors begin calling within days; most are wrong about what the survivor owes, but the conversations are intimidating and the rules vary by state. The available resources are accurate and encyclopedic; they list eighty things the executor might need to do, with no way to know which twelve apply today.
+**Users.** The executor — spouse, adult child, or sibling — grieving and doing this because someone had to be. Institutions and debt collectors are stakeholders, not the design's target. Scope is from the first week through final dissolution.
+**Cost.** The work runs in the evenings on top of grief, on top of a job, on top of a household that did not pause. The encyclopedic list does not tell the executor which twelve of eighty steps belong to today, so the wrong ones get done first or none at all. The collectors' calls keep coming. The estate stays open, the mail keeps arriving, and the grief is interrupted every time the ordeal reasserts itself.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -875,14 +851,10 @@
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t># Driver's license transfer after a cross-state move — design exploration
-## Situation
-A person has moved from one US state to another. They have a job to start, an apartment to unpack, a kid in a new school. Somewhere on the list is "transfer the driver's license," and the new state's DMV site is a tangle of pages that don't quite match the user's situation: out-of-state transfer vs new resident vs non-citizen vs recently-licensed teen. They have a stack of documents — birth certificate, Social Security card, lease, utility bill, old license, marriage certificate.
-## Complication
-They aren't sure which documents the office will accept on the day. They want to know when to go, what to bring, what the visit will feel like, and what happens if something goes wrong. The DMV won't tell them ahead of time. The mover does the visit, leaves with a temporary paper printout, and waits weeks for the hard copy in the mail. In the meantime they aren't sure whether the paper is enough to fly, open a bank account, or pass any other ID check.
-## Users
-A recent mover in the four-to-six-week window after a cross-state move, navigating the new state's DMV alone with a folder of documents and other life on fire.
-## Cost
-Getting any of this wrong costs another visit, another day of work missed, and the same lack of information about what's next. The scope is the four-to-six-week window after a move during which the license needs to transfer.</t>
+**Situation.** A person has moved from one US state to another. They have a job to start, an apartment to unpack, a kid in a new school. Somewhere on the list is "transfer the driver's license," and the new state's DMV site is a tangle of pages that don't quite match the user's situation: out-of-state transfer vs new resident vs non-citizen vs recently-licensed teen. They have a stack of documents — birth certificate, Social Security card, lease, utility bill, old license, marriage certificate.
+**Complication.** They aren't sure which documents the office will accept on the day. They want to know when to go, what to bring, what the visit will feel like, and what happens if something goes wrong. The DMV won't tell them ahead of time. The mover does the visit, leaves with a temporary paper printout, and waits weeks for the hard copy in the mail. In the meantime they aren't sure whether the paper is enough to fly, open a bank account, or pass any other ID check.
+**Users.** A recent mover in the four-to-six-week window after a cross-state move, navigating the new state's DMV alone with a folder of documents and other life on fire.
+**Cost.** Getting any of this wrong costs another visit, another day of work missed, and the same lack of information about what's next. The scope is the four-to-six-week window after a move during which the license needs to transfer.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -935,14 +907,10 @@
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t># A first-time manager's first performance review — design exploration
-## Situation
-Someone who has been a people manager for less than a year sits down at midnight to write their first performance review of an employee. They have nine weeks of notes — most of them mental — and a template HR handed down with fifteen sections and a five-point rating scale. They are also navigating a calibration cycle in which their ratings will be compared against peer managers' ratings, with rules they only half-understand.
-## Complication
-The performance-management software they're using delivers prompts and templates but does not actually help them think through what to say to this specific person about this specific thing. They are scared of doing harm. Of giving feedback that lands wrong. Of being too soft and ducking the real issue. Of being too critical and damaging a working relationship. They are alone with a form and a blinking cursor.
-## Users
-A first-time people manager writing their first review of a direct report — who might be a former peer, someone they hired, or someone with more years in the industry than they have. HR and the calibration committee are stakeholders the manager has to satisfy, but the design is for the manager in the moment of writing.
-## Cost
-The cost of getting this wrong is paid both at the next 1:1 and across the year that follows — a damaged working relationship, a real issue ducked, or feedback that lands so wrong it forecloses growth. The scope is the act of writing the review — the hours between *I have to write this* and *I have a draft I'd send.*</t>
+**Situation.** Someone who has been a people manager for less than a year sits down at midnight to write their first performance review of an employee. They have nine weeks of notes — most of them mental — and a template HR handed down with fifteen sections and a five-point rating scale. They are also navigating a calibration cycle in which their ratings will be compared against peer managers' ratings, with rules they only half-understand.
+**Complication.** The performance-management software they're using delivers prompts and templates but does not actually help them think through what to say to this specific person about this specific thing. They are scared of doing harm. Of giving feedback that lands wrong. Of being too soft and ducking the real issue. Of being too critical and damaging a working relationship. They are alone with a form and a blinking cursor.
+**Users.** A first-time people manager writing their first review of a direct report — who might be a former peer, someone they hired, or someone with more years in the industry than they have. HR and the calibration committee are stakeholders the manager has to satisfy, but the design is for the manager in the moment of writing.
+**Cost.** The cost of getting this wrong is paid both at the next 1:1 and across the year that follows — a damaged working relationship, a real issue ducked, or feedback that lands so wrong it forecloses growth. The scope is the act of writing the review — the hours between *I have to write this* and *I have a draft I'd send.*</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -996,14 +964,10 @@
       <c r="B10" s="3" t="inlineStr">
         <is>
           <t># A grief-focused web app — design exploration
-## Situation
-We're scoping a web product for people in active grief. The space today splits roughly three ways: funeral logistics sites (transactional, mostly pre-funeral), peer support communities and subreddits (exposing or noisy for many), and journaling apps that bolt on a "feeling sad" mood tag (toothless). The users we keep hearing from describe wanting something different — something that respects them as someone grieving rather than treating them as a user to be moved through a funnel or a feed.
-## Complication
-People reach for a tool at the awkward moments: 3am, the anniversary, after a hard conversation with a sibling about settling the estate, on a Tuesday for no specific reason. At those moments, the funeral sites read transactional, the subreddits feel either welcoming or hostile depending on luck, and the mood-tag prompt asks "how are you feeling today?" as if grief were a state to log. Existing tools fail them by being too prescriptive ("step 4 of 7: write a letter to your loved one") or too generic.
-## Users
-Anyone weeks-to-months out from a meaningful loss — recent enough that grief is shaping the day, not so recent that they're still in funeral logistics. The losses vary: parent, partner, friend, pregnancy, pet, anticipatory loss with a terminal diagnosis. The support systems around them vary more — some surrounded by attentive friends, others whose network has gone quiet at six weeks.
-## Cost
-The cost of failure isn't dramatic — it's the slow drift away from a tool that doesn't meet them, and the continued absence of a place that does. What we want from this round: distinct strategic directions for what "a web app for grief" could meaningfully be — real bets that could move the category, not convergent variants.</t>
+**Situation.** We're scoping a web product for people in active grief. The space today splits roughly three ways: funeral logistics sites (transactional, mostly pre-funeral), peer support communities and subreddits (exposing or noisy for many), and journaling apps that bolt on a "feeling sad" mood tag (toothless). The users we keep hearing from describe wanting something different — something that respects them as someone grieving rather than treating them as a user to be moved through a funnel or a feed.
+**Complication.** People reach for a tool at the awkward moments: 3am, the anniversary, after a hard conversation with a sibling about settling the estate, on a Tuesday for no specific reason. At those moments, the funeral sites read transactional, the subreddits feel either welcoming or hostile depending on luck, and the mood-tag prompt asks "how are you feeling today?" as if grief were a state to log. Existing tools fail them by being too prescriptive ("step 4 of 7: write a letter to your loved one") or too generic.
+**Users.** Anyone weeks-to-months out from a meaningful loss — recent enough that grief is shaping the day, not so recent that they're still in funeral logistics. The losses vary: parent, partner, friend, pregnancy, pet, anticipatory loss with a terminal diagnosis. The support systems around them vary more — some surrounded by attentive friends, others whose network has gone quiet at six weeks.
+**Cost.** The cost of failure isn't dramatic — it's the slow drift away from a tool that doesn't meet them, and the continued absence of a place that does. What we want from this round: distinct strategic directions for what "a web app for grief" could meaningfully be — real bets that could move the category, not convergent variants.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1058,14 +1022,10 @@
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t># Discharge instructions for older adults going home — design exploration
-## Situation
-An older adult is being discharged from the hospital this afternoon after a heart-failure exacerbation, a stroke, a fall, or pneumonia. A family caregiver — often an adult child who has travelled in — will run the first week or two at home. The nurse has roughly fifteen minutes to walk through six pages of paperwork before the next admission needs the room.
-## Complication
-The patient is in pain, on medications that affect cognition, exhausted and emotionally activated; what they remember of those fifteen minutes once home is fragmentary. The caregiver who will administer the next thirty days is sometimes in the room and sometimes not. A few days later, the patient is trying to figure out which white pill is the new beta-blocker, what "weigh yourself daily and call if you gain more than three pounds in a week" means in practice, whether today's ankle swelling is a warning sign, and what the printed phone number is for after hours. The discharge papers are face-down on the kitchen table next to the medication bottles. The follow-up is in eleven days.
-## Users
-The dyad post-discharge: the older adult patient recovering at home, and the family caregiver — often an adult child — running the first week or two of medications, warning signs, and follow-up logistics. The discharging nurse and follow-up clinic are stakeholders the design accommodates; the design is for the dyad once paperwork has come home.
-## Cost
-Between now and the follow-up, it is the patient and the caregiver and the paperwork. The cost of getting it wrong is a missed warning sign, a doubled medication, a readmission. Scope is the discharge moment plus the first 7–14 days at home; the clinical care plan is out of scope.</t>
+**Situation.** An older adult is being discharged from the hospital this afternoon after a heart-failure exacerbation, a stroke, a fall, or pneumonia. A family caregiver — often an adult child who has travelled in — will run the first week or two at home. The nurse has roughly fifteen minutes to walk through six pages of paperwork before the next admission needs the room.
+**Complication.** The patient is in pain, on medications that affect cognition, exhausted and emotionally activated; what they remember of those fifteen minutes once home is fragmentary. The caregiver who will administer the next thirty days is sometimes in the room and sometimes not. A few days later, the patient is trying to figure out which white pill is the new beta-blocker, what "weigh yourself daily and call if you gain more than three pounds in a week" means in practice, whether today's ankle swelling is a warning sign, and what the printed phone number is for after hours. The discharge papers are face-down on the kitchen table next to the medication bottles. The follow-up is in eleven days.
+**Users.** The dyad post-discharge: the older adult patient recovering at home, and the family caregiver — often an adult child — running the first week or two of medications, warning signs, and follow-up logistics. The discharging nurse and follow-up clinic are stakeholders the design accommodates; the design is for the dyad once paperwork has come home.
+**Cost.** Between now and the follow-up, it is the patient and the caregiver and the paperwork. The cost of getting it wrong is a missed warning sign, a doubled medication, a readmission. Scope is the discharge moment plus the first 7–14 days at home; the clinical care plan is out of scope.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1122,14 +1082,10 @@
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t># Self-representation in housing court — design exploration
-## Situation
-A tenant has received an eviction notice. Their landlord has filed in housing court. They have a court date in two to three weeks. They cannot afford an attorney; the legal-aid clinic in their county is at capacity. The available self-help resources are accurate, thorough, and unusable in their situation: long PDFs of legalese for someone who is working two jobs and putting kids to bed at the same time.
-## Complication
-The tenant may or may not have a legal defense. The landlord may not have given proper notice; the rent claim may be wrong; the unit may be uninhabitable; the landlord may have engaged in unlawful self-help. Or the tenant may not have a defense and needs to negotiate time, settle, or simply file an answer to preserve options. They have a stack of papers in three different formats, a phone, and an internet connection. They cannot tell which of the eighty pieces of available advice apply to their facts and which don't.
-## Users
-A pro-se tenant facing an eviction filing with a court date two to three weeks out, navigating the case alone. Legal-aid attorneys, court clerks, and the landlord's counsel are stakeholders the tenant encounters; the design is for the tenant doing the work between notice and hearing.
-## Cost
-What they need is to walk into court understanding what is about to happen and what they should say. The cost of falling short is a default judgment, a lost home, and a record that follows them to the next lease application. The scope is from "I got a notice" through "I have prepared for court."</t>
+**Situation.** A tenant has received an eviction notice. Their landlord has filed in housing court. They have a court date in two to three weeks. They cannot afford an attorney; the legal-aid clinic in their county is at capacity. The available self-help resources are accurate, thorough, and unusable in their situation: long PDFs of legalese for someone who is working two jobs and putting kids to bed at the same time.
+**Complication.** The tenant may or may not have a legal defense. The landlord may not have given proper notice; the rent claim may be wrong; the unit may be uninhabitable; the landlord may have engaged in unlawful self-help. Or the tenant may not have a defense and needs to negotiate time, settle, or simply file an answer to preserve options. They have a stack of papers in three different formats, a phone, and an internet connection. They cannot tell which of the eighty pieces of available advice apply to their facts and which don't.
+**Users.** A pro-se tenant facing an eviction filing with a court date two to three weeks out, navigating the case alone. Legal-aid attorneys, court clerks, and the landlord's counsel are stakeholders the tenant encounters; the design is for the tenant doing the work between notice and hearing.
+**Cost.** What they need is to walk into court understanding what is about to happen and what they should say. The cost of falling short is a default judgment, a lost home, and a record that follows them to the next lease application. The scope is from "I got a notice" through "I have prepared for court."</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1184,14 +1140,10 @@
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t># Multi-currency expense report submission — design exploration
-## Situation
-A traveler is home for two days between business trips. The trip that just ended ran through three countries, with receipts in five formats, photos of meals in a foreign language, an airline charge that hit their card in USD but was billed in EUR, a hotel charge pre-authorized at one amount and posted at another, an Uber auto-uploaded but mis-categorized as personal, and a cash tip paid because the card terminal was broken. They have policy questions — was the upgraded flight reimbursable, what counts as a client meal — and no one to ask quickly.
-## Complication
-They submit. Finance rejects it for a single category mismatch and asks them to redo. Each round of back-and-forth is another evening they don't have. The available expense tools present categorization screens, FX-rate prompts, and approval flows; the gap between what the traveler can produce on a Saturday afternoon and what finance needs to approve is where the loop lives.
-## Users
-The business traveler reconciling between trips — competent, time-starved, working from a kitchen table with a phone full of receipts. The finance reviewer reads what was submitted and often sends it back; they are a stakeholder, not the target.
-## Cost
-Evenings lost to resubmissions, the next trip approaching with last trip's report still open, reimbursements that lag for weeks, and the slow erosion of any sense that this part of the job is tractable. The traveler is leaving for São Paulo on Sunday. The scope is from the moment a trip ends to the moment the report is approved.</t>
+**Situation.** A traveler is home for two days between business trips. The trip that just ended ran through three countries, with receipts in five formats, photos of meals in a foreign language, an airline charge that hit their card in USD but was billed in EUR, a hotel charge pre-authorized at one amount and posted at another, an Uber auto-uploaded but mis-categorized as personal, and a cash tip paid because the card terminal was broken. They have policy questions — was the upgraded flight reimbursable, what counts as a client meal — and no one to ask quickly.
+**Complication.** They submit. Finance rejects it for a single category mismatch and asks them to redo. Each round of back-and-forth is another evening they don't have. The available expense tools present categorization screens, FX-rate prompts, and approval flows; the gap between what the traveler can produce on a Saturday afternoon and what finance needs to approve is where the loop lives.
+**Users.** The business traveler reconciling between trips — competent, time-starved, working from a kitchen table with a phone full of receipts. The finance reviewer reads what was submitted and often sends it back; they are a stakeholder, not the target.
+**Cost.** Evenings lost to resubmissions, the next trip approaching with last trip's report still open, reimbursements that lag for weeks, and the slow erosion of any sense that this part of the job is tractable. The traveler is leaving for São Paulo on Sunday. The scope is from the moment a trip ends to the moment the report is approved.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1247,14 +1199,10 @@
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t># A parent finding tutoring for a child struggling in math — design exploration
-## Situation
-A child in 4th, 6th, or 8th grade is struggling in math. The grades have slipped; the teacher has sent a note; the standardized test result came back lower than expected. The parent has a few hours over the next two weeks to set something up, working evenings around their own job and the rest of the family's calendar.
-## Complication
-The parent is facing a tangle of options the landscape currently presents: the local tutoring chain (predictable but expensive, small-group, weekly); a private tutor matched through a friend (variable quality and availability); online tutoring marketplaces and free practice platforms; the school's own intervention program if the kid qualifies; AI-tutor apps that promise personalization. The parent cannot easily tell which option is matched to what works versus what's marketing. They are not the math expert.
-## Users
-A parent–child dyad at the moment of choosing help. The parent is the procurer and decider — scheduling, paying, reading reviews, judging fit. The child is the recipient and the one whose engagement determines whether any of this works; they are sensitive to the framing, since *you need a tutor* can feel like a judgment, and a kid who closes off doesn't learn from anyone. Tutor candidates and school staff are stakeholders the design accommodates, not the target.
-## Cost
-Weeks pass while the parent stalls between bad options; the child falls further behind in a subject that compounds; the wrong choice burns money and the child's willingness to try again. The scope is from "we need help" through "we have a plan and a tutor we trust."</t>
+**Situation.** A child in 4th, 6th, or 8th grade is struggling in math. The grades have slipped; the teacher has sent a note; the standardized test result came back lower than expected. The parent has a few hours over the next two weeks to set something up, working evenings around their own job and the rest of the family's calendar.
+**Complication.** The parent is facing a tangle of options the landscape currently presents: the local tutoring chain (predictable but expensive, small-group, weekly); a private tutor matched through a friend (variable quality and availability); online tutoring marketplaces and free practice platforms; the school's own intervention program if the kid qualifies; AI-tutor apps that promise personalization. The parent cannot easily tell which option is matched to what works versus what's marketing. They are not the math expert.
+**Users.** A parent–child dyad at the moment of choosing help. The parent is the procurer and decider — scheduling, paying, reading reviews, judging fit. The child is the recipient and the one whose engagement determines whether any of this works; they are sensitive to the framing, since *you need a tutor* can feel like a judgment, and a kid who closes off doesn't learn from anyone. Tutor candidates and school staff are stakeholders the design accommodates, not the target.
+**Cost.** Weeks pass while the parent stalls between bad options; the child falls further behind in a subject that compounds; the wrong choice burns money and the child's willingness to try again. The scope is from "we need help" through "we have a plan and a tutor we trust."</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1309,14 +1257,10 @@
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t># Pre-travel prescription preparation — design exploration
-## Situation
-A person is preparing for a long international trip. They take regular prescription medication — an SSRI, an ADHD stimulant, a blood thinner, hormone therapy, a controlled-substance painkiller. They are two weeks out and just realized this is harder than they thought. US prescriptions can't be filled at overseas pharmacies. Several common US medications are restricted or illegal in the country they're going to.
-## Complication
-To carry enough for the trip, they need a vacation override from their insurance, weeks in advance, and probably a prescriber letter. None of that is one phone call. They are working it out across pharmacy phone trees, the insurer's app, the State Department's site, and Reddit threads. Their PCP's office is not set up to answer travel-medication questions. The pharmacy can fill the script if the doctor authorizes the override; the doctor will authorize the override if asked correctly. Nobody owns the work of getting this person across the world with their medication intact, legal, and packaged the way customs expects.
-## Users
-An international traveler on regular, often controlled, prescription medication — a person managing real conditions who needs to keep managing them on the other side of a border. Prescriber, pharmacist, insurer, and customs are stakeholders this work moves through, not the target.
-## Cost
-Consequences run from confiscation at customs to denial of entry to arrest in stricter jurisdictions, plus the quieter failure of running out of medication mid-trip and the destabilization that follows. The scope is the four-week window before international departure.</t>
+**Situation.** A person is preparing for a long international trip. They take regular prescription medication — an SSRI, an ADHD stimulant, a blood thinner, hormone therapy, a controlled-substance painkiller. They are two weeks out and just realized this is harder than they thought. US prescriptions can't be filled at overseas pharmacies. Several common US medications are restricted or illegal in the country they're going to.
+**Complication.** To carry enough for the trip, they need a vacation override from their insurance, weeks in advance, and probably a prescriber letter. None of that is one phone call. They are working it out across pharmacy phone trees, the insurer's app, the State Department's site, and Reddit threads. Their PCP's office is not set up to answer travel-medication questions. The pharmacy can fill the script if the doctor authorizes the override; the doctor will authorize the override if asked correctly. Nobody owns the work of getting this person across the world with their medication intact, legal, and packaged the way customs expects.
+**Users.** An international traveler on regular, often controlled, prescription medication — a person managing real conditions who needs to keep managing them on the other side of a border. Prescriber, pharmacist, insurer, and customs are stakeholders this work moves through, not the target.
+**Cost.** Consequences run from confiscation at customs to denial of entry to arrest in stricter jurisdictions, plus the quieter failure of running out of medication mid-trip and the destabilization that follows. The scope is the four-week window before international departure.</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1356,14 +1300,10 @@
       <c r="B16" s="3" t="inlineStr">
         <is>
           <t># Finding a primary care doctor after relocating — design exploration
-## Situation
-A person has moved to a new city and needs a primary care doctor. They have insurance, and their plan's website hands them an in-network directory — several hundred names, sorted by ZIP code. The directory shows specialties and addresses. It rarely shows which practices are accepting new patients, what the next available appointment actually is, which clinicians speak the languages spoken in the patient's household, whether the office is wheelchair-accessible, or how the practice handles diabetes care, mental-health needs, or pregnancy.
-## Complication
-The patient calls one office, sits on hold for ten minutes, navigates a phone tree, and is told the next opening is in five months — or that the practice isn't accepting new patients at all. Then the next call. Then the next. The options they are choosing between in the landscape today include the in-network directory itself, telehealth services their plan covers, federally-qualified health centers in the area, and direct primary care practices that bill outside insurance — none of which the directory surfaces side-by-side.
-## Users
-A patient looking for a primary care doctor in a new city. Some have active conditions — chronic pain, diabetes, anxiety — and need to start care now; others are establishing routine care and re-engage only when something goes wrong. The insurance plan, the in-network directory, the practices, and telehealth providers are stakeholder context the design accommodates, not the target.
-## Cost
-Delayed care for people who need it now; undiagnosed conditions for those who give up early; emergency visits for what should have been clinic visits. The scope is from "I need a new doctor" through "I have an appointment booked."</t>
+**Situation.** A person has moved to a new city and needs a primary care doctor. They have insurance, and their plan's website hands them an in-network directory — several hundred names, sorted by ZIP code. The directory shows specialties and addresses. It rarely shows which practices are accepting new patients, what the next available appointment actually is, which clinicians speak the languages spoken in the patient's household, whether the office is wheelchair-accessible, or how the practice handles diabetes care, mental-health needs, or pregnancy.
+**Complication.** The patient calls one office, sits on hold for ten minutes, navigates a phone tree, and is told the next opening is in five months — or that the practice isn't accepting new patients at all. Then the next call. Then the next. The options they are choosing between in the landscape today include the in-network directory itself, telehealth services their plan covers, federally-qualified health centers in the area, and direct primary care practices that bill outside insurance — none of which the directory surfaces side-by-side.
+**Users.** A patient looking for a primary care doctor in a new city. Some have active conditions — chronic pain, diabetes, anxiety — and need to start care now; others are establishing routine care and re-engage only when something goes wrong. The insurance plan, the in-network directory, the practices, and telehealth providers are stakeholder context the design accommodates, not the target.
+**Cost.** Delayed care for people who need it now; undiagnosed conditions for those who give up early; emergency visits for what should have been clinic visits. The scope is from "I need a new doctor" through "I have an appointment booked."</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1404,14 +1344,10 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t># Remote new-hire onboarding, week one — design exploration
-## Situation
-A competent professional joins a remote-first company on Monday. They have never met their team in person. They've done this before — they know how to set up a laptop and learn a new codebase. The HR-built first week is nine meetings Monday, six Tuesday; a stack of documentation; a Notion they still can't fully access; benefits links, security trainings, and a Slack workspace with a hundred channels.
-## Complication
-What's hard isn't the work; it's everything around it. They don't know this team's norms, this manager's actual (not stated) preferences, who is the person you actually ask about benefits. Remote replaces the watercooler, the lunch tag-along, and the overheard standup with calendar invites — which aren't the same thing. By Wednesday the orientation rush slows; by Thursday they're alone with documentation and unsure who to ask what, anxious about asking questions that would mark them as not-yet-onboard.
-## Users
-The new hire — a competent professional starting cold inside a remote-first company, navigating their first five working days from a home desk. The hiring manager, peers on the team, HR, and IT provisioning are stakeholders whose work shapes the week but who are not the target of the design.
-## Cost
-The five-day window from joining to belonging is where the relationship is made or lost; new hires who don't feel onboard by Friday carry that uncertainty into the next month, hesitate to ask, and quietly disengage. Companies bleed early-tenure hires at exactly this point. The scope is the first five working days, Monday morning to Friday afternoon.</t>
+**Situation.** A competent professional joins a remote-first company on Monday. They have never met their team in person. They've done this before — they know how to set up a laptop and learn a new codebase. The HR-built first week is nine meetings Monday, six Tuesday; a stack of documentation; a Notion they still can't fully access; benefits links, security trainings, and a Slack workspace with a hundred channels.
+**Complication.** What's hard isn't the work; it's everything around it. They don't know this team's norms, this manager's actual (not stated) preferences, who is the person you actually ask about benefits. Remote replaces the watercooler, the lunch tag-along, and the overheard standup with calendar invites — which aren't the same thing. By Wednesday the orientation rush slows; by Thursday they're alone with documentation and unsure who to ask what, anxious about asking questions that would mark them as not-yet-onboard.
+**Users.** The new hire — a competent professional starting cold inside a remote-first company, navigating their first five working days from a home desk. The hiring manager, peers on the team, HR, and IT provisioning are stakeholders whose work shapes the week but who are not the target of the design.
+**Cost.** The five-day window from joining to belonging is where the relationship is made or lost; new hires who don't feel onboard by Friday carry that uncertainty into the next month, hesitate to ask, and quietly disengage. Companies bleed early-tenure hires at exactly this point. The scope is the first five working days, Monday morning to Friday afternoon.</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1466,14 +1402,10 @@
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t># A sprint retro after a missed target — design exploration
-## Situation
-A product team has just finished a two-week sprint and missed what they committed to. The scrum master has forty-five minutes booked on Friday afternoon for the retrospective. The team is tired, the engineer who carried the cancelled feature is quiet on the call, the PM is reading their phone, and the VP of Engineering is on the line listening in. The scrum master has a Miro board with three columns and a stack of sticky notes their team has used in some version for the last two years.
-## Complication
-The team's existing tools — Miro templates, FunRetro, EasyRetro, the Jira retro module — capture sticky notes and let people upvote them. What happens between "sticky notes captured" and "the team had a real conversation" sits outside those tools. The team itself is uneven: some members will say what they think directly, some won't say anything that could read as criticism with the PM in the room, and some will narrate the sprint as if it went fine.
-## Users
-The scrum master is the target user — the one prepping the meeting, holding the room, and chasing follow-through. The team is the design's audience; the PM in the room and the VP listening in are stakeholders the meeting accommodates.
-## Cost
-A retro that doesn't land after a missed sprint compounds: the same patterns carry into the next sprint, action items are forgotten by Monday, and the team grows a little more cynical about whether retros are worth showing up to. A retro that does land is something the team can feel for weeks. The scope is the retrospective meeting itself, the prep before it, and the follow-through.</t>
+**Situation.** A product team has just finished a two-week sprint and missed what they committed to. The scrum master has forty-five minutes booked on Friday afternoon for the retrospective. The team is tired, the engineer who carried the cancelled feature is quiet on the call, the PM is reading their phone, and the VP of Engineering is on the line listening in. The scrum master has a Miro board with three columns and a stack of sticky notes their team has used in some version for the last two years.
+**Complication.** The team's existing tools — Miro templates, FunRetro, EasyRetro, the Jira retro module — capture sticky notes and let people upvote them. What happens between "sticky notes captured" and "the team had a real conversation" sits outside those tools. The team itself is uneven: some members will say what they think directly, some won't say anything that could read as criticism with the PM in the room, and some will narrate the sprint as if it went fine.
+**Users.** The scrum master is the target user — the one prepping the meeting, holding the room, and chasing follow-through. The team is the design's audience; the PM in the room and the VP listening in are stakeholders the meeting accommodates.
+**Cost.** A retro that doesn't land after a missed sprint compounds: the same patterns carry into the next sprint, action items are forgotten by Monday, and the team grows a little more cynical about whether retros are worth showing up to. A retro that does land is something the team can feel for weeks. The scope is the retrospective meeting itself, the prep before it, and the follow-through.</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1514,14 +1446,10 @@
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t># Applying for food assistance — design exploration
-## Situation
-Someone who needs food assistance now is sitting down to apply for SNAP. They've lost a job, had hours cut, gotten sick, or are raising a kid on inconsistent income. They are working from a phone, sometimes a shared one, often on intermittent data.
-## Complication
-The form in front of them asks branching questions whose answers depend on context the form does not let them explain, requires documents they can't easily produce in the moment (a recent pay stub from a gig that pays inconsistently, a lease they don't have a copy of, a Social Security card from a drawer at a place they no longer live), and was built to be filled out on a desktop computer they don't own. After they submit, the experience goes quiet. They don't know if the application was received, is being processed, is waiting on a document the system has not asked for, or has already been denied.
-## Users
-The target user is the applicant: a first-time applicant who has never used the safety net, a mixed-status family weighing whether the application itself will be used against them, or someone returning under worse circumstances than the first time. State eligibility workers who process and adjudicate these applications are stakeholders, not the target.
-## Cost
-Days pass. The food situation that brought them here doesn't pause. Many people in this position get one attempt before they stop trying — not from a single rejection, but from the cumulative weight of submitting into silence while the rest of their life keeps moving. What we want: distinct strategic directions for what a humane food-assistance application could be when designed around the applicant.</t>
+**Situation.** Someone who needs food assistance now is sitting down to apply for SNAP. They've lost a job, had hours cut, gotten sick, or are raising a kid on inconsistent income. They are working from a phone, sometimes a shared one, often on intermittent data.
+**Complication.** The form in front of them asks branching questions whose answers depend on context the form does not let them explain, requires documents they can't easily produce in the moment (a recent pay stub from a gig that pays inconsistently, a lease they don't have a copy of, a Social Security card from a drawer at a place they no longer live), and was built to be filled out on a desktop computer they don't own. After they submit, the experience goes quiet. They don't know if the application was received, is being processed, is waiting on a document the system has not asked for, or has already been denied.
+**Users.** The target user is the applicant: a first-time applicant who has never used the safety net, a mixed-status family weighing whether the application itself will be used against them, or someone returning under worse circumstances than the first time. State eligibility workers who process and adjudicate these applications are stakeholders, not the target.
+**Cost.** Days pass. The food situation that brought them here doesn't pause. Many people in this position get one attempt before they stop trying — not from a single rejection, but from the cumulative weight of submitting into silence while the rest of their life keeps moving. What we want: distinct strategic directions for what a humane food-assistance application could be when designed around the applicant.</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1576,14 +1504,10 @@
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t># The first 90 days after a Type 2 diabetes diagnosis — design exploration
-## Situation
-A person has just been told they have Type 2 diabetes. The diagnosis arrived in a fifteen-minute appointment with a handout, a prescription for metformin, and instructions to "watch your sugars" and to "see a nutritionist." They walk out scared, ashamed, confused about whether they caused this, and facing a slate of changes — diet, exercise, medication, glucose monitoring, A1c labs every three months.
-## Complication
-No one helps them sequence those changes. The nutritionist referral is a phone number on the printout. The diabetes self-management education and support sessions their insurance covers are not mentioned at the appointment. The landscape they encounter when they look for help — glucose-logging utilities, coaching platforms (Livongo, Virta, Omada), peer-support communities, and YouTube videos from creators of varying authority — tends to ask them to log their glucose on day one. None of it is shaped around the moment of diagnosis itself: the week they are still telling family, the week they are deciding whether to tell work.
-## Users
-The target user is the newly-diagnosed patient in the first 90 days. The clinician and the nutritionist are stakeholders the design accommodates — referrals come from them, labs route through them — but are not who the design is for.
-## Cost
-By the end of the next ninety days they will have either built a workable rhythm — meals, walking, the morning metformin, the glucose meter sitting on the kitchen counter — or they will have drifted: meter in a drawer, prescription unfilled at refill time, weight unchanged, and no further appointment booked until the next labs flag something. The scope is from diagnosis through the 90-day mark.</t>
+**Situation.** A person has just been told they have Type 2 diabetes. The diagnosis arrived in a fifteen-minute appointment with a handout, a prescription for metformin, and instructions to "watch your sugars" and to "see a nutritionist." They walk out scared, ashamed, confused about whether they caused this, and facing a slate of changes — diet, exercise, medication, glucose monitoring, A1c labs every three months.
+**Complication.** No one helps them sequence those changes. The nutritionist referral is a phone number on the printout. The diabetes self-management education and support sessions their insurance covers are not mentioned at the appointment. The landscape they encounter when they look for help — glucose-logging utilities, coaching platforms (Livongo, Virta, Omada), peer-support communities, and YouTube videos from creators of varying authority — tends to ask them to log their glucose on day one. None of it is shaped around the moment of diagnosis itself: the week they are still telling family, the week they are deciding whether to tell work.
+**Users.** The target user is the newly-diagnosed patient in the first 90 days. The clinician and the nutritionist are stakeholders the design accommodates — referrals come from them, labs route through them — but are not who the design is for.
+**Cost.** By the end of the next ninety days they will have either built a workable rhythm — meals, walking, the morning metformin, the glucose meter sitting on the kitchen counter — or they will have drifted: meter in a drawer, prescription unfilled at refill time, weight unchanged, and no further appointment booked until the next labs flag something. The scope is from diagnosis through the 90-day mark.</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1623,14 +1547,10 @@
       <c r="B21" s="3" t="inlineStr">
         <is>
           <t># Filing for unemployment insurance — design exploration
-## Situation
-A person has just lost their job and is filing for unemployment insurance through their state's labor agency. They may have a few weeks of rent in the bank or none. They are filling out the application on a phone — in line at a job center, between caregiving shifts, or late at night after the kids are asleep.
-## Complication
-The application asks for an EDDCAN number they have never heard of, pay stubs from the last eighteen months they may not have saved, and the precise dates and hours of every job worked in a base period that doesn't match how variable-schedule work happens. The legalese is dense. A wrong answer on any of dozens of questions delays or denies the claim, and the appeal that follows takes weeks. Once filed, the channels for finding out what's happening are a state portal that often shows information weeks out of date, paper letters that arrive after the next pay period would have been due, and a phone line that holds for hours. The portal sometimes says the claim is being processed; sometimes nothing at all.
-## Users
-The target user is the claimant — filing and waiting on benefits they are entitled to under state and federal law. State eligibility workers and adjudicators are stakeholders, not the target.
-## Cost
-Money does not arrive on a schedule the person can plan around. Rent is due, the car insurance lapses, the kid needs school supplies. The gap between filing and the first payment landing is where the urgency of the situation collides with what the system communicates. The scope is the filing flow plus the first thirty days of claim-status communication.</t>
+**Situation.** A person has just lost their job and is filing for unemployment insurance through their state's labor agency. They may have a few weeks of rent in the bank or none. They are filling out the application on a phone — in line at a job center, between caregiving shifts, or late at night after the kids are asleep.
+**Complication.** The application asks for an EDDCAN number they have never heard of, pay stubs from the last eighteen months they may not have saved, and the precise dates and hours of every job worked in a base period that doesn't match how variable-schedule work happens. The legalese is dense. A wrong answer on any of dozens of questions delays or denies the claim, and the appeal that follows takes weeks. Once filed, the channels for finding out what's happening are a state portal that often shows information weeks out of date, paper letters that arrive after the next pay period would have been due, and a phone line that holds for hours. The portal sometimes says the claim is being processed; sometimes nothing at all.
+**Users.** The target user is the claimant — filing and waiting on benefits they are entitled to under state and federal law. State eligibility workers and adjudicators are stakeholders, not the target.
+**Cost.** Money does not arrive on a schedule the person can plan around. Rent is due, the car insurance lapses, the kid needs school supplies. The gap between filing and the first payment landing is where the urgency of the situation collides with what the system communicates. The scope is the filing flow plus the first thirty days of claim-status communication.</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1670,14 +1590,10 @@
       <c r="B22" s="3" t="inlineStr">
         <is>
           <t># Updating voter registration after a name change — design exploration
-## Situation
-A person has changed their legal name — after marriage, divorce, gender transition, leaving an abusive relationship, or by personal choice. Their old name is on the voter roll. The next election is months away. Someone told them they should update their registration; they don't know whether they need to, by when, what proof, or how their state's rules differ from a friend's in another state.
-## Complication
-The state election-board website is a tangle of pages and PDFs that don't quite match their situation. Voter registration sits inside a long list of bureaucratic to-dos the name change has triggered — driver's license, Social Security card, employer records, banking, passports — and is the one most likely to be skipped until election day.
-## Users
-The target user is the voter mid-name-change: a trans person whose ID is finally catching up to their name, a domestic-violence survivor who changed their name for safety, a recently-married or recently-divorced voter, or someone who chose a new name. Each comes with different proof, different timelines, and different concerns about who sees the old name during the update. Election-board staff and poll workers are stakeholders, not the target.
-## Cost
-On election day, the name fails the poll-book check and they're asked to cast a provisional ballot they may not return to cure. A vote they were entitled to cast doesn't count, and being challenged at the table — especially for trans voters or survivors whose old name is read aloud — can make them less likely to return. The scope is updating registration plus the ambiguity around it — *do I need to, when by, what proof, will this be wrong on election day.*</t>
+**Situation.** A person has changed their legal name — after marriage, divorce, gender transition, leaving an abusive relationship, or by personal choice. Their old name is on the voter roll. The next election is months away. Someone told them they should update their registration; they don't know whether they need to, by when, what proof, or how their state's rules differ from a friend's in another state.
+**Complication.** The state election-board website is a tangle of pages and PDFs that don't quite match their situation. Voter registration sits inside a long list of bureaucratic to-dos the name change has triggered — driver's license, Social Security card, employer records, banking, passports — and is the one most likely to be skipped until election day.
+**Users.** The target user is the voter mid-name-change: a trans person whose ID is finally catching up to their name, a domestic-violence survivor who changed their name for safety, a recently-married or recently-divorced voter, or someone who chose a new name. Each comes with different proof, different timelines, and different concerns about who sees the old name during the update. Election-board staff and poll workers are stakeholders, not the target.
+**Cost.** On election day, the name fails the poll-book check and they're asked to cast a provisional ballot they may not return to cure. A vote they were entitled to cast doesn't count, and being challenged at the table — especially for trans voters or survivors whose old name is read aloud — can make them less likely to return. The scope is updating registration plus the ambiguity around it — *do I need to, when by, what proof, will this be wrong on election day.*</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">

</xml_diff>